<commit_message>
Auto-place SL order 20 points below entry for intraday 9:20
Feature: When placing BUY order via /api/intraday-920/place-order:
1. Place BUY order at market price
2. If BUY succeeds, automatically place SL order
3. SL trigger price = Entry Price - 20 points
4. SL order placed with same lot size as entry

Response includes:
- order_id: BUY order ID
- sl_order_id: SL order ID (if successful)
- sl_trigger_price: SL price (entry - 20)
- sl_success: Whether SL was placed successfully
- sl_error: Error message if SL placement failed

Example:
- Entry: 101 at 105
- SL: 85 (105 - 20)
- Both orders placed automatically in one API call
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:P58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3140,6 +3140,232 @@
       <c r="P53" s="2" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 13:40:00</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>13:40:00</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>78.25</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>198.95</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr"/>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 13:40:00</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>13:40:00</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>155.00</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>99.00</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr"/>
+      <c r="L55" s="2" t="inlineStr"/>
+      <c r="M55" s="2" t="inlineStr"/>
+      <c r="N55" s="2" t="inlineStr"/>
+      <c r="O55" s="2" t="inlineStr"/>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 13:45:00</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>13:45:00</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr"/>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr"/>
+      <c r="O56" s="2" t="inlineStr"/>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 13:50:00</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>13:50:00</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr"/>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr"/>
+      <c r="O57" s="2" t="inlineStr"/>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 13:55:00</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>13:55:00</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr"/>
+      <c r="M58" s="2" t="inlineStr"/>
+      <c r="N58" s="2" t="inlineStr"/>
+      <c r="O58" s="2" t="inlineStr"/>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Auto-place SL order - correct entry price extraction and add detailed logging
Issues Fixed:
1. Changed entry_price to price (actual field returned by place_order)
2. Added comprehensive error logging for each step
3. Add validation for entry_price > 0
4. Return early if entry_price is invalid

Logging Added:
- [SL] prefix for all stoploss-related logs
- Log option_symbol retrieval
- Log lot size retrieval
- Log SL order placement attempt
- Log SL order result
- Log all errors with context

Response Format:
- sl_order_id: SL order ID (if successful)
- sl_trigger_price: SL trigger price
- sl_success: true/false
- sl_error: Error message if failed

Now SL orders should auto-place correctly after BUY orders
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P58"/>
+  <dimension ref="A1:P60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3366,6 +3366,106 @@
       <c r="P58" s="2" t="inlineStr">
         <is>
           <t>Failed to fetch data: Live data fetch timed out after 10s</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 14:00:00</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>78.25</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>198.95</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="2" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr"/>
+      <c r="O59" s="2" t="inlineStr"/>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 14:00:00</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>155.00</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>99.00</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr"/>
+      <c r="M60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr"/>
+      <c r="O60" s="2" t="inlineStr"/>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Stoploss order price tick size alignment - resolve Zerodha error 16283
Problem: 'Order price is not a multiple of tick size' error
- Zerodha options require prices aligned to 0.05 (5 paise) tick size
- Previous calculation (trigger_price * 0.998) created invalid prices
- Example: 85.50 * 0.998 = 85.323 (invalid, not multiple of 0.05)

Solution: Round execution price to proper tick size
1. TICK_SIZE = 0.05 (5 paise for index options)
2. Round DOWN to nearest tick: int(price / 0.05) * 0.05
3. Ensure execution_price is below trigger price
4. Final validation rounding to 2 decimals

Example:
- Trigger: 85.50 (multiple of 0.05 ✓)
- Execution: 85.45 (multiple of 0.05 ✓)
- Both valid tick-aligned prices

Affects: All stoploss orders for intraday 9:20 strategy
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P60"/>
+  <dimension ref="A1:P61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3466,6 +3466,48 @@
       <c r="P60" s="2" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 14:05:00</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>14:05:00</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr"/>
+      <c r="O61" s="2" t="inlineStr"/>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Improve Fyers authentication error handling and documentation
- Enhanced error message in /auth/login/fyers with clear instructions
- Shows which credentials are missing (APP_ID vs SECRET_KEY)
- Provides link to Fyers Dashboard for credential retrieval
- Updated env templates with correct field name FYERS_SECRET_KEY
- Standardized comments in env files
- Added comprehensive FYERS_SETUP.md guide for configuration
- Explains step-by-step how to get and configure credentials
- Includes troubleshooting section for common issues
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1543,6 +1543,248 @@
       <c r="P21" s="6" t="inlineStr">
         <is>
           <t>Failed to fetch data: Live data fetch timed out after 10s</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 09:30:00</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr"/>
+      <c r="K22" s="6" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr"/>
+      <c r="M22" s="6" t="inlineStr"/>
+      <c r="N22" s="6" t="inlineStr"/>
+      <c r="O22" s="6" t="inlineStr"/>
+      <c r="P22" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 09:30:00</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr"/>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr"/>
+      <c r="K23" s="6" t="inlineStr"/>
+      <c r="L23" s="6" t="inlineStr"/>
+      <c r="M23" s="6" t="inlineStr"/>
+      <c r="N23" s="6" t="inlineStr"/>
+      <c r="O23" s="6" t="inlineStr"/>
+      <c r="P23" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 09:35:00</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>09:35:00</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr"/>
+      <c r="F24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr"/>
+      <c r="K24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr"/>
+      <c r="M24" s="6" t="inlineStr"/>
+      <c r="N24" s="6" t="inlineStr"/>
+      <c r="O24" s="6" t="inlineStr"/>
+      <c r="P24" s="6" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 09:35:00</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>09:35:00</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr"/>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr"/>
+      <c r="K25" s="6" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr"/>
+      <c r="M25" s="6" t="inlineStr"/>
+      <c r="N25" s="6" t="inlineStr"/>
+      <c r="O25" s="6" t="inlineStr"/>
+      <c r="P25" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 09:35:00</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>09:35:00</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr"/>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr"/>
+      <c r="K26" s="6" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr"/>
+      <c r="M26" s="6" t="inlineStr"/>
+      <c r="N26" s="6" t="inlineStr"/>
+      <c r="O26" s="6" t="inlineStr"/>
+      <c r="P26" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Correct variable naming and import paths from live data refactoring
- Fix: Change undefined 'max_retries' to 'max_date_retries' in intraday_9_20.py (lines 191, 194)
  - Variable was renamed during retry logic restructuring but references weren't updated
- Fix: Move NetworkException/TokenException import to correct path in kite_order_services.py
  - Change: from kiteconnect import → from kiteconnect.exceptions import
  - Ensures proper exception handling in get_current_prices_batch()

These were caught by workspace error validation after previous implementation.
All syntax errors now cleared.
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P42"/>
+  <dimension ref="A1:P44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2551,6 +2551,106 @@
       <c r="N42" s="6" t="inlineStr"/>
       <c r="O42" s="6" t="inlineStr"/>
       <c r="P42" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 10:30:00</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr"/>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr"/>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J43" s="6" t="inlineStr"/>
+      <c r="K43" s="6" t="inlineStr"/>
+      <c r="L43" s="6" t="inlineStr"/>
+      <c r="M43" s="6" t="inlineStr"/>
+      <c r="N43" s="6" t="inlineStr"/>
+      <c r="O43" s="6" t="inlineStr"/>
+      <c r="P43" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 10:30:00</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr"/>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr"/>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J44" s="6" t="inlineStr"/>
+      <c r="K44" s="6" t="inlineStr"/>
+      <c r="L44" s="6" t="inlineStr"/>
+      <c r="M44" s="6" t="inlineStr"/>
+      <c r="N44" s="6" t="inlineStr"/>
+      <c r="O44" s="6" t="inlineStr"/>
+      <c r="P44" s="6" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>

</xml_diff>

<commit_message>
fix: Optimize candle fetching to prevent timeout errors
IMPROVEMENTS:
1. Increase live data fetch timeout from 20s to 45s
   - Allows sufficient time for candle fetching with retries
   - Better accommodates slow API responses during peak hours

2. Optimize candle retry loop: 30 days → 3 days max
   - Most trades happen within last 2 trading days
   - Reduces API calls and prevents excessive retries
   - Faster fallback logic

3. Better timeout error messaging
   - Now indicates it's the candle fetching taking too long
   - Will retry on next 5-minute cycle

RATIONALE:
- 20s timeout was too short when fetching CE and PE candles in parallel
- Each candle fetch with connection retry can take 3-8 seconds
- 45s total gives proper buffer for all operations to complete
- Reduced retry days from 30 to 3 cuts unnecessary API calls

EXPECTED RESULT:
- Fewer timeout errors during peak hours (11:00 - 14:00)
- Faster response times by avoiding excessive retries
- More stable live data fetching
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -33,7 +33,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -58,19 +58,28 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -112,10 +121,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -483,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P44"/>
+  <dimension ref="A1:P53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -579,950 +588,982 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:05:00</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>13:05:00</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>13:05</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>155.00</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>99.00</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-10 10:50:00</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>10:50:00</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="n"/>
+      <c r="K2" s="5" t="n"/>
+      <c r="L2" s="5" t="n"/>
+      <c r="M2" s="5" t="n"/>
+      <c r="N2" s="5" t="n"/>
+      <c r="O2" s="5" t="n"/>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-10 10:50:00</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>10:50:00</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="n"/>
+      <c r="K3" s="5" t="n"/>
+      <c r="L3" s="5" t="n"/>
+      <c r="M3" s="5" t="n"/>
+      <c r="N3" s="5" t="n"/>
+      <c r="O3" s="5" t="n"/>
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:10:00</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>13:10:00</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>13:10</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>78.25</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>198.95</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
-      <c r="O3" s="2" t="n"/>
-      <c r="P3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 10:55:00</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>10:55:00</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr"/>
+      <c r="K4" s="6" t="inlineStr"/>
+      <c r="L4" s="6" t="inlineStr"/>
+      <c r="M4" s="6" t="inlineStr"/>
+      <c r="N4" s="6" t="inlineStr"/>
+      <c r="O4" s="6" t="inlineStr"/>
+      <c r="P4" s="6" t="inlineStr">
         <is>
           <t>High Strike Check</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:10:00</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>13:10:00</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>13:10</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>155.00</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>99.00</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="n"/>
-      <c r="O4" s="2" t="n"/>
-      <c r="P4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 10:55:00</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>10:55:00</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="6" t="inlineStr"/>
+      <c r="N5" s="6" t="inlineStr"/>
+      <c r="O5" s="6" t="inlineStr"/>
+      <c r="P5" s="6" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:15:00</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>13:15:00</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>13:15</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>78.25</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>198.95</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="n"/>
-      <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="n"/>
-      <c r="O5" s="2" t="n"/>
-      <c r="P5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:00:00</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>11:00:00</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
+      <c r="L6" s="6" t="inlineStr"/>
+      <c r="M6" s="6" t="inlineStr"/>
+      <c r="N6" s="6" t="inlineStr"/>
+      <c r="O6" s="6" t="inlineStr"/>
+      <c r="P6" s="6" t="inlineStr">
         <is>
           <t>High Strike Check</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:15:00</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>13:15:00</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>13:15</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>155.00</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>99.00</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="n"/>
-      <c r="O6" s="2" t="n"/>
-      <c r="P6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:00:00</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>11:00:00</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:20:00</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>13:20:00</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>13:20</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
-        </is>
-      </c>
-    </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:35:00</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>13:35:00</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>13:35</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>155.00</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>198.95</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>✓ YES</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>104.80</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:05:00</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>11:05:00</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr"/>
+      <c r="M8" s="6" t="inlineStr"/>
+      <c r="N8" s="6" t="inlineStr"/>
+      <c r="O8" s="6" t="inlineStr"/>
+      <c r="P8" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:05:00</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>11:05:00</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>79.00</t>
         </is>
       </c>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>156.40</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="n"/>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="inlineStr"/>
+      <c r="P9" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:10:00</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>11:10:00</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
+      <c r="M10" s="6" t="inlineStr"/>
+      <c r="N10" s="6" t="inlineStr"/>
+      <c r="O10" s="6" t="inlineStr"/>
+      <c r="P10" s="6" t="inlineStr">
         <is>
           <t>High Strike Check</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:35:00</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>13:35:00</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>13:35</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>155.00</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>99.00</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>✓ YES</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>104.80</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:10:00</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>11:10:00</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>79.00</t>
         </is>
       </c>
-      <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>156.40</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="n"/>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
+      <c r="M11" s="6" t="inlineStr"/>
+      <c r="N11" s="6" t="inlineStr"/>
+      <c r="O11" s="6" t="inlineStr"/>
+      <c r="P11" s="6" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:40:00</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>13:40:00</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>13:40</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>78.25</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>198.95</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
-      <c r="O10" s="2" t="n"/>
-      <c r="P10" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:15:00</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>11:15:00</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
+      <c r="M12" s="6" t="inlineStr"/>
+      <c r="N12" s="6" t="inlineStr"/>
+      <c r="O12" s="6" t="inlineStr"/>
+      <c r="P12" s="6" t="inlineStr">
         <is>
           <t>High Strike Check</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:40:00</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>13:40:00</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>13:40</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>155.00</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>99.00</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="n"/>
-      <c r="O11" s="2" t="n"/>
-      <c r="P11" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:15:00</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>11:15:00</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr"/>
+      <c r="M13" s="6" t="inlineStr"/>
+      <c r="N13" s="6" t="inlineStr"/>
+      <c r="O13" s="6" t="inlineStr"/>
+      <c r="P13" s="6" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:45:00</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>13:45:00</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>13:45</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="n"/>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="n"/>
-      <c r="O12" s="2" t="n"/>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:50:00</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>13:50:00</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>13:50</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
-      <c r="O13" s="2" t="n"/>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
-        </is>
-      </c>
-    </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 13:55:00</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>13:55:00</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>13:55</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="n"/>
-      <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="n"/>
-      <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="n"/>
-      <c r="O14" s="2" t="n"/>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:20:00</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>11:20:00</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr"/>
+      <c r="K14" s="6" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr"/>
+      <c r="M14" s="6" t="inlineStr"/>
+      <c r="N14" s="6" t="inlineStr"/>
+      <c r="O14" s="6" t="inlineStr"/>
+      <c r="P14" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 14:00:00</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>14:00:00</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>78.25</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>198.95</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="n"/>
-      <c r="K15" s="2" t="n"/>
-      <c r="L15" s="2" t="n"/>
-      <c r="M15" s="2" t="n"/>
-      <c r="N15" s="2" t="n"/>
-      <c r="O15" s="2" t="n"/>
-      <c r="P15" s="2" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:20:00</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>11:20:00</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr"/>
+      <c r="M15" s="6" t="inlineStr"/>
+      <c r="N15" s="6" t="inlineStr"/>
+      <c r="O15" s="6" t="inlineStr"/>
+      <c r="P15" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:25:00</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>11:25:00</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr"/>
+      <c r="K16" s="6" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr"/>
+      <c r="M16" s="6" t="inlineStr"/>
+      <c r="N16" s="6" t="inlineStr"/>
+      <c r="O16" s="6" t="inlineStr"/>
+      <c r="P16" s="6" t="inlineStr">
         <is>
           <t>High Strike Check</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 14:00:00</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>14:00:00</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>155.00</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>99.00</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="n"/>
-      <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="n"/>
-      <c r="M16" s="2" t="n"/>
-      <c r="N16" s="2" t="n"/>
-      <c r="O16" s="2" t="n"/>
-      <c r="P16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:25:00</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>11:25:00</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="inlineStr"/>
+      <c r="N17" s="6" t="inlineStr"/>
+      <c r="O17" s="6" t="inlineStr"/>
+      <c r="P17" s="6" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 14:05:00</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>14:05:00</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>14:05</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="n"/>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="n"/>
-      <c r="O17" s="2" t="n"/>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
-        </is>
-      </c>
-    </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-10 09:15:00</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>09:15:00</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>09:15</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:30:00</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>11:30:00</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>83.70</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>111.10</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="n"/>
-      <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
-      <c r="M18" s="2" t="n"/>
-      <c r="N18" s="2" t="n"/>
-      <c r="O18" s="2" t="n"/>
-      <c r="P18" s="2" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr"/>
+      <c r="K18" s="6" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr"/>
+      <c r="M18" s="6" t="inlineStr"/>
+      <c r="N18" s="6" t="inlineStr"/>
+      <c r="O18" s="6" t="inlineStr"/>
+      <c r="P18" s="6" t="inlineStr">
         <is>
           <t>High Strike Check</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-10 09:15:00</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>09:15:00</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>09:15</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>130.00</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>34.00</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="n"/>
-      <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="n"/>
-      <c r="N19" s="2" t="n"/>
-      <c r="O19" s="2" t="n"/>
-      <c r="P19" s="2" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:30:00</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>11:30:00</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr"/>
+      <c r="K19" s="6" t="inlineStr"/>
+      <c r="L19" s="6" t="inlineStr"/>
+      <c r="M19" s="6" t="inlineStr"/>
+      <c r="N19" s="6" t="inlineStr"/>
+      <c r="O19" s="6" t="inlineStr"/>
+      <c r="P19" s="6" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-10 09:20:00</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>09:20:00</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>09:20</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>✗ NO</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>Failed to fetch data: Error fetching quote: ('Connection aborted.', ConnectionResetError(54, 'Connection reset by peer'))</t>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 11:35:00</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>11:35:00</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr"/>
+      <c r="K20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr"/>
+      <c r="M20" s="6" t="inlineStr"/>
+      <c r="N20" s="6" t="inlineStr"/>
+      <c r="O20" s="6" t="inlineStr"/>
+      <c r="P20" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:25:00</t>
+          <t>2026-02-10 11:35:00</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>09:25:00</t>
+          <t>11:35:00</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>09:25</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr"/>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
       <c r="E21" s="6" t="inlineStr"/>
-      <c r="F21" s="6" t="inlineStr"/>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr">
         <is>
@@ -1542,24 +1583,24 @@
       <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
+          <t>Low Strike Check</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:30:00</t>
+          <t>2026-02-10 11:40:00</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>09:30:00</t>
+          <t>11:40:00</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -1599,17 +1640,17 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:30:00</t>
+          <t>2026-02-10 11:40:00</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>09:30:00</t>
+          <t>11:40:00</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1649,22 +1690,30 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:35:00</t>
+          <t>2026-02-10 11:45:00</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>09:35:00</t>
+          <t>11:45:00</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>09:35</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr"/>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
       <c r="E24" s="6" t="inlineStr"/>
-      <c r="F24" s="6" t="inlineStr"/>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
       <c r="G24" s="6" t="inlineStr"/>
       <c r="H24" s="6" t="inlineStr">
         <is>
@@ -1684,35 +1733,35 @@
       <c r="O24" s="6" t="inlineStr"/>
       <c r="P24" s="6" t="inlineStr">
         <is>
-          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
+          <t>High Strike Check</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:35:00</t>
+          <t>2026-02-10 11:45:00</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>09:35:00</t>
+          <t>11:45:00</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>83.70</t>
+          <t>102.00</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr"/>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>111.75</t>
+          <t>79.00</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr"/>
@@ -1734,35 +1783,35 @@
       <c r="O25" s="6" t="inlineStr"/>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>High Strike Check</t>
+          <t>Low Strike Check</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:35:00</t>
+          <t>2026-02-10 11:50:00</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>09:35:00</t>
+          <t>11:50:00</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>11:50</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>102.00</t>
+          <t>83.70</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr"/>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>79.00</t>
+          <t>111.75</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr"/>
@@ -1784,29 +1833,37 @@
       <c r="O26" s="6" t="inlineStr"/>
       <c r="P26" s="6" t="inlineStr">
         <is>
-          <t>Low Strike Check</t>
+          <t>High Strike Check</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:40:00</t>
+          <t>2026-02-10 11:50:00</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>09:40:00</t>
+          <t>11:50:00</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>09:40</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr"/>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
       <c r="E27" s="6" t="inlineStr"/>
-      <c r="F27" s="6" t="inlineStr"/>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
       <c r="G27" s="6" t="inlineStr"/>
       <c r="H27" s="6" t="inlineStr">
         <is>
@@ -1826,29 +1883,37 @@
       <c r="O27" s="6" t="inlineStr"/>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
+          <t>Low Strike Check</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:45:00</t>
+          <t>2026-02-10 11:55:00</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>09:45:00</t>
+          <t>11:55:00</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>09:45</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr"/>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
       <c r="E28" s="6" t="inlineStr"/>
-      <c r="F28" s="6" t="inlineStr"/>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
       <c r="G28" s="6" t="inlineStr"/>
       <c r="H28" s="6" t="inlineStr">
         <is>
@@ -1868,35 +1933,35 @@
       <c r="O28" s="6" t="inlineStr"/>
       <c r="P28" s="6" t="inlineStr">
         <is>
-          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
+          <t>High Strike Check</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:50:00</t>
+          <t>2026-02-10 11:55:00</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>09:50:00</t>
+          <t>11:55:00</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>09:50</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>83.70</t>
+          <t>102.00</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr"/>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>111.75</t>
+          <t>79.00</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr"/>
@@ -1918,35 +1983,35 @@
       <c r="O29" s="6" t="inlineStr"/>
       <c r="P29" s="6" t="inlineStr">
         <is>
-          <t>High Strike Check</t>
+          <t>Low Strike Check</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:50:00</t>
+          <t>2026-02-10 12:00:00</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>09:50:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>09:50</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>102.00</t>
+          <t>83.70</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr"/>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>79.00</t>
+          <t>111.75</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr"/>
@@ -1968,35 +2033,35 @@
       <c r="O30" s="6" t="inlineStr"/>
       <c r="P30" s="6" t="inlineStr">
         <is>
-          <t>Low Strike Check</t>
+          <t>High Strike Check</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:55:00</t>
+          <t>2026-02-10 12:00:00</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>09:55:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>83.70</t>
+          <t>102.00</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr"/>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>111.75</t>
+          <t>79.00</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr"/>
@@ -2018,37 +2083,29 @@
       <c r="O31" s="6" t="inlineStr"/>
       <c r="P31" s="6" t="inlineStr">
         <is>
-          <t>High Strike Check</t>
+          <t>Low Strike Check</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 09:55:00</t>
+          <t>2026-02-10 12:05:00</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>09:55:00</t>
+          <t>12:05:00</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>09:55</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>102.00</t>
-        </is>
-      </c>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr"/>
       <c r="E32" s="6" t="inlineStr"/>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>79.00</t>
-        </is>
-      </c>
+      <c r="F32" s="6" t="inlineStr"/>
       <c r="G32" s="6" t="inlineStr"/>
       <c r="H32" s="6" t="inlineStr">
         <is>
@@ -2068,29 +2125,37 @@
       <c r="O32" s="6" t="inlineStr"/>
       <c r="P32" s="6" t="inlineStr">
         <is>
-          <t>Low Strike Check</t>
+          <t>Failed to fetch data: Live data fetch timed out after 20s - possible API or network issue</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:00:00</t>
+          <t>2026-02-10 12:10:00</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:10:00</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr"/>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
       <c r="E33" s="6" t="inlineStr"/>
-      <c r="F33" s="6" t="inlineStr"/>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
       <c r="G33" s="6" t="inlineStr"/>
       <c r="H33" s="6" t="inlineStr">
         <is>
@@ -2110,29 +2175,37 @@
       <c r="O33" s="6" t="inlineStr"/>
       <c r="P33" s="6" t="inlineStr">
         <is>
-          <t>Failed to fetch data: Live data fetch timed out after 10s</t>
+          <t>High Strike Check</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:05:00</t>
+          <t>2026-02-10 12:10:00</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>10:05:00</t>
+          <t>12:10:00</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>10:05</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr"/>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
       <c r="E34" s="6" t="inlineStr"/>
-      <c r="F34" s="6" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
       <c r="G34" s="6" t="inlineStr"/>
       <c r="H34" s="6" t="inlineStr">
         <is>
@@ -2152,37 +2225,29 @@
       <c r="O34" s="6" t="inlineStr"/>
       <c r="P34" s="6" t="inlineStr">
         <is>
-          <t>Failed to fetch data: Error fetching quote: ('Connection aborted.', ConnectionResetError(54, 'Connection reset by peer'))</t>
+          <t>Low Strike Check</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:10:00</t>
+          <t>2026-02-10 12:15:00</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>10:10:00</t>
+          <t>12:15:00</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>10:10</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>83.70</t>
-        </is>
-      </c>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr"/>
       <c r="E35" s="6" t="inlineStr"/>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>111.75</t>
-        </is>
-      </c>
+      <c r="F35" s="6" t="inlineStr"/>
       <c r="G35" s="6" t="inlineStr"/>
       <c r="H35" s="6" t="inlineStr">
         <is>
@@ -2202,35 +2267,35 @@
       <c r="O35" s="6" t="inlineStr"/>
       <c r="P35" s="6" t="inlineStr">
         <is>
-          <t>High Strike Check</t>
+          <t>Failed to fetch data: Live data fetch timed out after 20s - possible API or network issue</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:10:00</t>
+          <t>2026-02-10 12:20:00</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>10:10:00</t>
+          <t>12:20:00</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>102.00</t>
+          <t>83.70</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr"/>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>79.00</t>
+          <t>111.75</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr"/>
@@ -2252,35 +2317,35 @@
       <c r="O36" s="6" t="inlineStr"/>
       <c r="P36" s="6" t="inlineStr">
         <is>
-          <t>Low Strike Check</t>
+          <t>High Strike Check</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:15:00</t>
+          <t>2026-02-10 12:20:00</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>10:15:00</t>
+          <t>12:20:00</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>83.70</t>
+          <t>102.00</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr"/>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>111.75</t>
+          <t>79.00</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr"/>
@@ -2302,35 +2367,35 @@
       <c r="O37" s="6" t="inlineStr"/>
       <c r="P37" s="6" t="inlineStr">
         <is>
-          <t>High Strike Check</t>
+          <t>Low Strike Check</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:15:00</t>
+          <t>2026-02-10 12:50:00</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>10:15:00</t>
+          <t>12:50:00</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>12:50</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>102.00</t>
+          <t>83.70</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr"/>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>79.00</t>
+          <t>111.75</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr"/>
@@ -2352,35 +2417,35 @@
       <c r="O38" s="6" t="inlineStr"/>
       <c r="P38" s="6" t="inlineStr">
         <is>
-          <t>Low Strike Check</t>
+          <t>High Strike Check</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:20:00</t>
+          <t>2026-02-10 12:50:00</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>10:20:00</t>
+          <t>12:50:00</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>12:50</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>83.70</t>
+          <t>102.00</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr"/>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>111.75</t>
+          <t>79.00</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr"/>
@@ -2402,37 +2467,29 @@
       <c r="O39" s="6" t="inlineStr"/>
       <c r="P39" s="6" t="inlineStr">
         <is>
-          <t>High Strike Check</t>
+          <t>Low Strike Check</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:20:00</t>
+          <t>2026-02-10 13:05:00</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>10:20:00</t>
+          <t>13:05:00</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>10:20</t>
-        </is>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>102.00</t>
-        </is>
-      </c>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr"/>
       <c r="E40" s="6" t="inlineStr"/>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>79.00</t>
-        </is>
-      </c>
+      <c r="F40" s="6" t="inlineStr"/>
       <c r="G40" s="6" t="inlineStr"/>
       <c r="H40" s="6" t="inlineStr">
         <is>
@@ -2452,24 +2509,24 @@
       <c r="O40" s="6" t="inlineStr"/>
       <c r="P40" s="6" t="inlineStr">
         <is>
-          <t>Low Strike Check</t>
+          <t>Failed to fetch data: Live data fetch timed out after 20s - possible API or network issue</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:25:00</t>
+          <t>2026-02-10 13:10:00</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>10:25:00</t>
+          <t>13:10:00</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -2509,17 +2566,17 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:25:00</t>
+          <t>2026-02-10 13:10:00</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>10:25:00</t>
+          <t>13:10:00</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
@@ -2559,17 +2616,17 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:30:00</t>
+          <t>2026-02-10 13:15:00</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>10:30:00</t>
+          <t>13:15:00</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
@@ -2609,17 +2666,17 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10 10:30:00</t>
+          <t>2026-02-10 13:15:00</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>10:30:00</t>
+          <t>13:15:00</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
@@ -2653,6 +2710,432 @@
       <c r="P44" s="6" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:20:00</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>13:20:00</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr"/>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J45" s="6" t="inlineStr"/>
+      <c r="K45" s="6" t="inlineStr"/>
+      <c r="L45" s="6" t="inlineStr"/>
+      <c r="M45" s="6" t="inlineStr"/>
+      <c r="N45" s="6" t="inlineStr"/>
+      <c r="O45" s="6" t="inlineStr"/>
+      <c r="P45" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:20:00</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>13:20:00</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr"/>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr"/>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="inlineStr"/>
+      <c r="K46" s="6" t="inlineStr"/>
+      <c r="L46" s="6" t="inlineStr"/>
+      <c r="M46" s="6" t="inlineStr"/>
+      <c r="N46" s="6" t="inlineStr"/>
+      <c r="O46" s="6" t="inlineStr"/>
+      <c r="P46" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:25:00</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>13:25:00</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr"/>
+      <c r="E47" s="6" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr"/>
+      <c r="G47" s="6" t="inlineStr"/>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J47" s="6" t="inlineStr"/>
+      <c r="K47" s="6" t="inlineStr"/>
+      <c r="L47" s="6" t="inlineStr"/>
+      <c r="M47" s="6" t="inlineStr"/>
+      <c r="N47" s="6" t="inlineStr"/>
+      <c r="O47" s="6" t="inlineStr"/>
+      <c r="P47" s="6" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Live data fetch timed out after 20s - possible API or network issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:30:00</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>13:30:00</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr"/>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr"/>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="inlineStr"/>
+      <c r="K48" s="6" t="inlineStr"/>
+      <c r="L48" s="6" t="inlineStr"/>
+      <c r="M48" s="6" t="inlineStr"/>
+      <c r="N48" s="6" t="inlineStr"/>
+      <c r="O48" s="6" t="inlineStr"/>
+      <c r="P48" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:30:00</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>13:30:00</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr"/>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr"/>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J49" s="6" t="inlineStr"/>
+      <c r="K49" s="6" t="inlineStr"/>
+      <c r="L49" s="6" t="inlineStr"/>
+      <c r="M49" s="6" t="inlineStr"/>
+      <c r="N49" s="6" t="inlineStr"/>
+      <c r="O49" s="6" t="inlineStr"/>
+      <c r="P49" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:35:00</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>13:35:00</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr"/>
+      <c r="E50" s="6" t="inlineStr"/>
+      <c r="F50" s="6" t="inlineStr"/>
+      <c r="G50" s="6" t="inlineStr"/>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="inlineStr"/>
+      <c r="K50" s="6" t="inlineStr"/>
+      <c r="L50" s="6" t="inlineStr"/>
+      <c r="M50" s="6" t="inlineStr"/>
+      <c r="N50" s="6" t="inlineStr"/>
+      <c r="O50" s="6" t="inlineStr"/>
+      <c r="P50" s="6" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Live data fetch timed out after 20s - possible API or network issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:40:00</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>13:40:00</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr"/>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr"/>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J51" s="6" t="inlineStr"/>
+      <c r="K51" s="6" t="inlineStr"/>
+      <c r="L51" s="6" t="inlineStr"/>
+      <c r="M51" s="6" t="inlineStr"/>
+      <c r="N51" s="6" t="inlineStr"/>
+      <c r="O51" s="6" t="inlineStr"/>
+      <c r="P51" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:40:00</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>13:40:00</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr"/>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr"/>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J52" s="6" t="inlineStr"/>
+      <c r="K52" s="6" t="inlineStr"/>
+      <c r="L52" s="6" t="inlineStr"/>
+      <c r="M52" s="6" t="inlineStr"/>
+      <c r="N52" s="6" t="inlineStr"/>
+      <c r="O52" s="6" t="inlineStr"/>
+      <c r="P52" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:45:00</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>13:45:00</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr"/>
+      <c r="E53" s="6" t="inlineStr"/>
+      <c r="F53" s="6" t="inlineStr"/>
+      <c r="G53" s="6" t="inlineStr"/>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="inlineStr"/>
+      <c r="K53" s="6" t="inlineStr"/>
+      <c r="L53" s="6" t="inlineStr"/>
+      <c r="M53" s="6" t="inlineStr"/>
+      <c r="N53" s="6" t="inlineStr"/>
+      <c r="O53" s="6" t="inlineStr"/>
+      <c r="P53" s="6" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Live data fetch timed out after 20s - possible API or network issue</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: Update logs and tokens
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -33,7 +33,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +56,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -125,6 +137,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -492,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:P89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3139,6 +3157,1854 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:50:00</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>13:50:00</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr"/>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr"/>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J54" s="6" t="inlineStr"/>
+      <c r="K54" s="6" t="inlineStr"/>
+      <c r="L54" s="6" t="inlineStr"/>
+      <c r="M54" s="6" t="inlineStr"/>
+      <c r="N54" s="6" t="inlineStr"/>
+      <c r="O54" s="6" t="inlineStr"/>
+      <c r="P54" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:50:00</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>13:50:00</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr"/>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr"/>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J55" s="6" t="inlineStr"/>
+      <c r="K55" s="6" t="inlineStr"/>
+      <c r="L55" s="6" t="inlineStr"/>
+      <c r="M55" s="6" t="inlineStr"/>
+      <c r="N55" s="6" t="inlineStr"/>
+      <c r="O55" s="6" t="inlineStr"/>
+      <c r="P55" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:55:00</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>13:55:00</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr"/>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr"/>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J56" s="6" t="inlineStr"/>
+      <c r="K56" s="6" t="inlineStr"/>
+      <c r="L56" s="6" t="inlineStr"/>
+      <c r="M56" s="6" t="inlineStr"/>
+      <c r="N56" s="6" t="inlineStr"/>
+      <c r="O56" s="6" t="inlineStr"/>
+      <c r="P56" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 13:55:00</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>13:55:00</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr"/>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr"/>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J57" s="6" t="inlineStr"/>
+      <c r="K57" s="6" t="inlineStr"/>
+      <c r="L57" s="6" t="inlineStr"/>
+      <c r="M57" s="6" t="inlineStr"/>
+      <c r="N57" s="6" t="inlineStr"/>
+      <c r="O57" s="6" t="inlineStr"/>
+      <c r="P57" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:00:00</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr"/>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr"/>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="inlineStr"/>
+      <c r="K58" s="6" t="inlineStr"/>
+      <c r="L58" s="6" t="inlineStr"/>
+      <c r="M58" s="6" t="inlineStr"/>
+      <c r="N58" s="6" t="inlineStr"/>
+      <c r="O58" s="6" t="inlineStr"/>
+      <c r="P58" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:00:00</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr"/>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr"/>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J59" s="6" t="inlineStr"/>
+      <c r="K59" s="6" t="inlineStr"/>
+      <c r="L59" s="6" t="inlineStr"/>
+      <c r="M59" s="6" t="inlineStr"/>
+      <c r="N59" s="6" t="inlineStr"/>
+      <c r="O59" s="6" t="inlineStr"/>
+      <c r="P59" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:05:00</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>14:05:00</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr"/>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr"/>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J60" s="6" t="inlineStr"/>
+      <c r="K60" s="6" t="inlineStr"/>
+      <c r="L60" s="6" t="inlineStr"/>
+      <c r="M60" s="6" t="inlineStr"/>
+      <c r="N60" s="6" t="inlineStr"/>
+      <c r="O60" s="6" t="inlineStr"/>
+      <c r="P60" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:05:00</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>14:05:00</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr"/>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr"/>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I61" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J61" s="6" t="inlineStr"/>
+      <c r="K61" s="6" t="inlineStr"/>
+      <c r="L61" s="6" t="inlineStr"/>
+      <c r="M61" s="6" t="inlineStr"/>
+      <c r="N61" s="6" t="inlineStr"/>
+      <c r="O61" s="6" t="inlineStr"/>
+      <c r="P61" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:10:00</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>14:10:00</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr"/>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr"/>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J62" s="6" t="inlineStr"/>
+      <c r="K62" s="6" t="inlineStr"/>
+      <c r="L62" s="6" t="inlineStr"/>
+      <c r="M62" s="6" t="inlineStr"/>
+      <c r="N62" s="6" t="inlineStr"/>
+      <c r="O62" s="6" t="inlineStr"/>
+      <c r="P62" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:10:00</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>14:10:00</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr"/>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr"/>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J63" s="6" t="inlineStr"/>
+      <c r="K63" s="6" t="inlineStr"/>
+      <c r="L63" s="6" t="inlineStr"/>
+      <c r="M63" s="6" t="inlineStr"/>
+      <c r="N63" s="6" t="inlineStr"/>
+      <c r="O63" s="6" t="inlineStr"/>
+      <c r="P63" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:15:00</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>14:15:00</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr"/>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr"/>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I64" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J64" s="6" t="inlineStr"/>
+      <c r="K64" s="6" t="inlineStr"/>
+      <c r="L64" s="6" t="inlineStr"/>
+      <c r="M64" s="6" t="inlineStr"/>
+      <c r="N64" s="6" t="inlineStr"/>
+      <c r="O64" s="6" t="inlineStr"/>
+      <c r="P64" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:15:00</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>14:15:00</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr"/>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr"/>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J65" s="6" t="inlineStr"/>
+      <c r="K65" s="6" t="inlineStr"/>
+      <c r="L65" s="6" t="inlineStr"/>
+      <c r="M65" s="6" t="inlineStr"/>
+      <c r="N65" s="6" t="inlineStr"/>
+      <c r="O65" s="6" t="inlineStr"/>
+      <c r="P65" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:20:00</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>14:20:00</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr"/>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr"/>
+      <c r="H66" s="8" t="inlineStr">
+        <is>
+          <t>✓ YES</t>
+        </is>
+      </c>
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J66" s="6" t="inlineStr">
+        <is>
+          <t>86.40</t>
+        </is>
+      </c>
+      <c r="K66" s="6" t="inlineStr"/>
+      <c r="L66" s="6" t="inlineStr">
+        <is>
+          <t>59.00</t>
+        </is>
+      </c>
+      <c r="M66" s="6" t="inlineStr"/>
+      <c r="N66" s="6" t="inlineStr">
+        <is>
+          <t>141.20</t>
+        </is>
+      </c>
+      <c r="O66" s="6" t="inlineStr"/>
+      <c r="P66" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:20:00</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>14:20:00</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr"/>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr"/>
+      <c r="H67" s="8" t="inlineStr">
+        <is>
+          <t>✓ YES</t>
+        </is>
+      </c>
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J67" s="6" t="inlineStr">
+        <is>
+          <t>86.40</t>
+        </is>
+      </c>
+      <c r="K67" s="6" t="inlineStr"/>
+      <c r="L67" s="6" t="inlineStr">
+        <is>
+          <t>59.00</t>
+        </is>
+      </c>
+      <c r="M67" s="6" t="inlineStr"/>
+      <c r="N67" s="6" t="inlineStr">
+        <is>
+          <t>141.20</t>
+        </is>
+      </c>
+      <c r="O67" s="6" t="inlineStr"/>
+      <c r="P67" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:25:00</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>14:25:00</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr"/>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr"/>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J68" s="6" t="inlineStr"/>
+      <c r="K68" s="6" t="inlineStr"/>
+      <c r="L68" s="6" t="inlineStr"/>
+      <c r="M68" s="6" t="inlineStr"/>
+      <c r="N68" s="6" t="inlineStr"/>
+      <c r="O68" s="6" t="inlineStr"/>
+      <c r="P68" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:25:00</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>14:25:00</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr"/>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr"/>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J69" s="6" t="inlineStr"/>
+      <c r="K69" s="6" t="inlineStr"/>
+      <c r="L69" s="6" t="inlineStr"/>
+      <c r="M69" s="6" t="inlineStr"/>
+      <c r="N69" s="6" t="inlineStr"/>
+      <c r="O69" s="6" t="inlineStr"/>
+      <c r="P69" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:30:00</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>14:30:00</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr"/>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr"/>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J70" s="6" t="inlineStr"/>
+      <c r="K70" s="6" t="inlineStr"/>
+      <c r="L70" s="6" t="inlineStr"/>
+      <c r="M70" s="6" t="inlineStr"/>
+      <c r="N70" s="6" t="inlineStr"/>
+      <c r="O70" s="6" t="inlineStr"/>
+      <c r="P70" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:30:00</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>14:30:00</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="inlineStr"/>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="inlineStr"/>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J71" s="6" t="inlineStr"/>
+      <c r="K71" s="6" t="inlineStr"/>
+      <c r="L71" s="6" t="inlineStr"/>
+      <c r="M71" s="6" t="inlineStr"/>
+      <c r="N71" s="6" t="inlineStr"/>
+      <c r="O71" s="6" t="inlineStr"/>
+      <c r="P71" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:35:00</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>14:35:00</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr"/>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr"/>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I72" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J72" s="6" t="inlineStr"/>
+      <c r="K72" s="6" t="inlineStr"/>
+      <c r="L72" s="6" t="inlineStr"/>
+      <c r="M72" s="6" t="inlineStr"/>
+      <c r="N72" s="6" t="inlineStr"/>
+      <c r="O72" s="6" t="inlineStr"/>
+      <c r="P72" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:35:00</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>14:35:00</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="inlineStr"/>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr"/>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J73" s="6" t="inlineStr"/>
+      <c r="K73" s="6" t="inlineStr"/>
+      <c r="L73" s="6" t="inlineStr"/>
+      <c r="M73" s="6" t="inlineStr"/>
+      <c r="N73" s="6" t="inlineStr"/>
+      <c r="O73" s="6" t="inlineStr"/>
+      <c r="P73" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:40:00</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>14:40:00</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr"/>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr"/>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J74" s="6" t="inlineStr"/>
+      <c r="K74" s="6" t="inlineStr"/>
+      <c r="L74" s="6" t="inlineStr"/>
+      <c r="M74" s="6" t="inlineStr"/>
+      <c r="N74" s="6" t="inlineStr"/>
+      <c r="O74" s="6" t="inlineStr"/>
+      <c r="P74" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:40:00</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>14:40:00</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr"/>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr"/>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J75" s="6" t="inlineStr"/>
+      <c r="K75" s="6" t="inlineStr"/>
+      <c r="L75" s="6" t="inlineStr"/>
+      <c r="M75" s="6" t="inlineStr"/>
+      <c r="N75" s="6" t="inlineStr"/>
+      <c r="O75" s="6" t="inlineStr"/>
+      <c r="P75" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:45:00</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr"/>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr"/>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J76" s="6" t="inlineStr"/>
+      <c r="K76" s="6" t="inlineStr"/>
+      <c r="L76" s="6" t="inlineStr"/>
+      <c r="M76" s="6" t="inlineStr"/>
+      <c r="N76" s="6" t="inlineStr"/>
+      <c r="O76" s="6" t="inlineStr"/>
+      <c r="P76" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:45:00</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr"/>
+      <c r="F77" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G77" s="6" t="inlineStr"/>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J77" s="6" t="inlineStr"/>
+      <c r="K77" s="6" t="inlineStr"/>
+      <c r="L77" s="6" t="inlineStr"/>
+      <c r="M77" s="6" t="inlineStr"/>
+      <c r="N77" s="6" t="inlineStr"/>
+      <c r="O77" s="6" t="inlineStr"/>
+      <c r="P77" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:50:00</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr"/>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr"/>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J78" s="6" t="inlineStr"/>
+      <c r="K78" s="6" t="inlineStr"/>
+      <c r="L78" s="6" t="inlineStr"/>
+      <c r="M78" s="6" t="inlineStr"/>
+      <c r="N78" s="6" t="inlineStr"/>
+      <c r="O78" s="6" t="inlineStr"/>
+      <c r="P78" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:50:00</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr"/>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G79" s="6" t="inlineStr"/>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J79" s="6" t="inlineStr"/>
+      <c r="K79" s="6" t="inlineStr"/>
+      <c r="L79" s="6" t="inlineStr"/>
+      <c r="M79" s="6" t="inlineStr"/>
+      <c r="N79" s="6" t="inlineStr"/>
+      <c r="O79" s="6" t="inlineStr"/>
+      <c r="P79" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:55:00</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>14:55:00</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr"/>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr"/>
+      <c r="H80" s="8" t="inlineStr">
+        <is>
+          <t>✓ YES</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J80" s="6" t="inlineStr">
+        <is>
+          <t>85.95</t>
+        </is>
+      </c>
+      <c r="K80" s="6" t="inlineStr"/>
+      <c r="L80" s="6" t="inlineStr">
+        <is>
+          <t>59.00</t>
+        </is>
+      </c>
+      <c r="M80" s="6" t="inlineStr"/>
+      <c r="N80" s="6" t="inlineStr">
+        <is>
+          <t>139.85</t>
+        </is>
+      </c>
+      <c r="O80" s="6" t="inlineStr"/>
+      <c r="P80" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:55:00</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>14:55:00</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr"/>
+      <c r="F81" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G81" s="6" t="inlineStr"/>
+      <c r="H81" s="8" t="inlineStr">
+        <is>
+          <t>✓ YES</t>
+        </is>
+      </c>
+      <c r="I81" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J81" s="6" t="inlineStr">
+        <is>
+          <t>85.95</t>
+        </is>
+      </c>
+      <c r="K81" s="6" t="inlineStr"/>
+      <c r="L81" s="6" t="inlineStr">
+        <is>
+          <t>59.00</t>
+        </is>
+      </c>
+      <c r="M81" s="6" t="inlineStr"/>
+      <c r="N81" s="6" t="inlineStr">
+        <is>
+          <t>139.85</t>
+        </is>
+      </c>
+      <c r="O81" s="6" t="inlineStr"/>
+      <c r="P81" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 15:00:00</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr"/>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G82" s="6" t="inlineStr"/>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="inlineStr"/>
+      <c r="K82" s="6" t="inlineStr"/>
+      <c r="L82" s="6" t="inlineStr"/>
+      <c r="M82" s="6" t="inlineStr"/>
+      <c r="N82" s="6" t="inlineStr"/>
+      <c r="O82" s="6" t="inlineStr"/>
+      <c r="P82" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 15:00:00</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr"/>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G83" s="6" t="inlineStr"/>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I83" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J83" s="6" t="inlineStr"/>
+      <c r="K83" s="6" t="inlineStr"/>
+      <c r="L83" s="6" t="inlineStr"/>
+      <c r="M83" s="6" t="inlineStr"/>
+      <c r="N83" s="6" t="inlineStr"/>
+      <c r="O83" s="6" t="inlineStr"/>
+      <c r="P83" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 15:05:00</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>15:05:00</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="inlineStr"/>
+      <c r="F84" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G84" s="6" t="inlineStr"/>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J84" s="6" t="inlineStr"/>
+      <c r="K84" s="6" t="inlineStr"/>
+      <c r="L84" s="6" t="inlineStr"/>
+      <c r="M84" s="6" t="inlineStr"/>
+      <c r="N84" s="6" t="inlineStr"/>
+      <c r="O84" s="6" t="inlineStr"/>
+      <c r="P84" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 15:05:00</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>15:05:00</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr"/>
+      <c r="F85" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G85" s="6" t="inlineStr"/>
+      <c r="H85" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I85" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J85" s="6" t="inlineStr"/>
+      <c r="K85" s="6" t="inlineStr"/>
+      <c r="L85" s="6" t="inlineStr"/>
+      <c r="M85" s="6" t="inlineStr"/>
+      <c r="N85" s="6" t="inlineStr"/>
+      <c r="O85" s="6" t="inlineStr"/>
+      <c r="P85" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 15:10:00</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>15:10:00</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="inlineStr"/>
+      <c r="F86" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G86" s="6" t="inlineStr"/>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I86" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J86" s="6" t="inlineStr"/>
+      <c r="K86" s="6" t="inlineStr"/>
+      <c r="L86" s="6" t="inlineStr"/>
+      <c r="M86" s="6" t="inlineStr"/>
+      <c r="N86" s="6" t="inlineStr"/>
+      <c r="O86" s="6" t="inlineStr"/>
+      <c r="P86" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 15:10:00</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>15:10:00</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr"/>
+      <c r="F87" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G87" s="6" t="inlineStr"/>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J87" s="6" t="inlineStr"/>
+      <c r="K87" s="6" t="inlineStr"/>
+      <c r="L87" s="6" t="inlineStr"/>
+      <c r="M87" s="6" t="inlineStr"/>
+      <c r="N87" s="6" t="inlineStr"/>
+      <c r="O87" s="6" t="inlineStr"/>
+      <c r="P87" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 15:15:00</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>15:15:00</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>83.70</t>
+        </is>
+      </c>
+      <c r="E88" s="6" t="inlineStr"/>
+      <c r="F88" s="6" t="inlineStr">
+        <is>
+          <t>111.75</t>
+        </is>
+      </c>
+      <c r="G88" s="6" t="inlineStr"/>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I88" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J88" s="6" t="inlineStr"/>
+      <c r="K88" s="6" t="inlineStr"/>
+      <c r="L88" s="6" t="inlineStr"/>
+      <c r="M88" s="6" t="inlineStr"/>
+      <c r="N88" s="6" t="inlineStr"/>
+      <c r="O88" s="6" t="inlineStr"/>
+      <c r="P88" s="6" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 15:15:00</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>15:15:00</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>102.00</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="inlineStr"/>
+      <c r="F89" s="6" t="inlineStr">
+        <is>
+          <t>79.00</t>
+        </is>
+      </c>
+      <c r="G89" s="6" t="inlineStr"/>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I89" s="6" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J89" s="6" t="inlineStr"/>
+      <c r="K89" s="6" t="inlineStr"/>
+      <c r="L89" s="6" t="inlineStr"/>
+      <c r="M89" s="6" t="inlineStr"/>
+      <c r="N89" s="6" t="inlineStr"/>
+      <c r="O89" s="6" t="inlineStr"/>
+      <c r="P89" s="6" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3150,7 +5016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3425,6 +5291,206 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:20:07</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>BUY CE</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>25850</v>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>86.40</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>86.40</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>BUY CE</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>2021144636487557120</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Mode: LIVE | Details: Order placed successfully via KiteService | Order_type: MARKET</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:20:08</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>SL_ORDER</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>25850</v>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>59.00</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>141.20</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>59.00</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>2021144641143234560</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>SL Order Placed | Trigger: 59.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:55:10</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>BUY CE</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>25850</v>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>85.95</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>85.95</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr"/>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>BUY CE</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>2021153458165833728</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>Mode: LIVE | Details: Order placed successfully via KiteService | Order_type: MARKET</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-10 14:55:11</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>SL_ORDER</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>25850</v>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>59.00</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>139.85</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>59.00</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>2021153462783762432</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>SL Order Placed | Trigger: 59.00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix OpenInterestService to fetch quotes from Kite API
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P63"/>
+  <dimension ref="A1:P67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3638,6 +3638,206 @@
       <c r="N63" s="4" t="inlineStr"/>
       <c r="O63" s="4" t="inlineStr"/>
       <c r="P63" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-11 14:45:00</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>146.45</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr"/>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>139.00</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr"/>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr"/>
+      <c r="K64" s="4" t="inlineStr"/>
+      <c r="L64" s="4" t="inlineStr"/>
+      <c r="M64" s="4" t="inlineStr"/>
+      <c r="N64" s="4" t="inlineStr"/>
+      <c r="O64" s="4" t="inlineStr"/>
+      <c r="P64" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-11 14:45:00</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>177.00</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>118.00</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr"/>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="inlineStr"/>
+      <c r="K65" s="4" t="inlineStr"/>
+      <c r="L65" s="4" t="inlineStr"/>
+      <c r="M65" s="4" t="inlineStr"/>
+      <c r="N65" s="4" t="inlineStr"/>
+      <c r="O65" s="4" t="inlineStr"/>
+      <c r="P65" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-11 14:50:00</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>146.45</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr"/>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>139.00</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr"/>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="inlineStr"/>
+      <c r="K66" s="4" t="inlineStr"/>
+      <c r="L66" s="4" t="inlineStr"/>
+      <c r="M66" s="4" t="inlineStr"/>
+      <c r="N66" s="4" t="inlineStr"/>
+      <c r="O66" s="4" t="inlineStr"/>
+      <c r="P66" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-11 14:50:00</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>177.00</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr"/>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>118.00</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr"/>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr"/>
+      <c r="K67" s="4" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr"/>
+      <c r="M67" s="4" t="inlineStr"/>
+      <c r="N67" s="4" t="inlineStr"/>
+      <c r="O67" s="4" t="inlineStr"/>
+      <c r="P67" s="4" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>

</xml_diff>

<commit_message>
♻️ Refactor OpenInterestService to reuse KiteService patterns
- Use _get_available_strikes() method similar to KiteDataFetchService
- Properly group instruments by strike with CE/PE tokens
- Filter to complete CE/PE pairs before fetching quotes
- Simplified logic reusing proven patterns from codebase
- Better error logging with all_names debug info
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P67"/>
+  <dimension ref="A1:P69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3838,6 +3838,106 @@
       <c r="N67" s="4" t="inlineStr"/>
       <c r="O67" s="4" t="inlineStr"/>
       <c r="P67" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-11 15:00:00</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>146.45</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr"/>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>139.00</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr"/>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr"/>
+      <c r="K68" s="4" t="inlineStr"/>
+      <c r="L68" s="4" t="inlineStr"/>
+      <c r="M68" s="4" t="inlineStr"/>
+      <c r="N68" s="4" t="inlineStr"/>
+      <c r="O68" s="4" t="inlineStr"/>
+      <c r="P68" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-11 15:00:00</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>177.00</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>118.00</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr"/>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr"/>
+      <c r="K69" s="4" t="inlineStr"/>
+      <c r="L69" s="4" t="inlineStr"/>
+      <c r="M69" s="4" t="inlineStr"/>
+      <c r="N69" s="4" t="inlineStr"/>
+      <c r="O69" s="4" t="inlineStr"/>
+      <c r="P69" s="4" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>

</xml_diff>

<commit_message>
🔧 Fix OpenInterestService - use direct dict key access instead of .get()
- Change from inst.get('name') to inst['name'] to match options_chart_service pattern
- Use try/except for safe key access instead of defensive .get()
- Cast strike to float and token to int for proper data types
- Add null checks with 'is not None' instead of falsy checks
- Add better error handling in quote fetch batches
- Log successful batch completions and quote counts
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P69"/>
+  <dimension ref="A1:P71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3938,6 +3938,106 @@
       <c r="N69" s="4" t="inlineStr"/>
       <c r="O69" s="4" t="inlineStr"/>
       <c r="P69" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-11 15:10:00</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>15:10:00</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>146.45</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr"/>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>139.00</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr"/>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr"/>
+      <c r="K70" s="4" t="inlineStr"/>
+      <c r="L70" s="4" t="inlineStr"/>
+      <c r="M70" s="4" t="inlineStr"/>
+      <c r="N70" s="4" t="inlineStr"/>
+      <c r="O70" s="4" t="inlineStr"/>
+      <c r="P70" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-11 15:10:00</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>15:10:00</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>177.00</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>118.00</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr"/>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr"/>
+      <c r="K71" s="4" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr"/>
+      <c r="M71" s="4" t="inlineStr"/>
+      <c r="N71" s="4" t="inlineStr"/>
+      <c r="O71" s="4" t="inlineStr"/>
+      <c r="P71" s="4" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>

</xml_diff>

<commit_message>
Fix opening OI cache initialization - handle all strike access paths
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1938,6 +1938,106 @@
       <c r="N29" s="4" t="inlineStr"/>
       <c r="O29" s="4" t="inlineStr"/>
       <c r="P29" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 10:20:00</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>10:20:00</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr"/>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr"/>
+      <c r="L30" s="4" t="inlineStr"/>
+      <c r="M30" s="4" t="inlineStr"/>
+      <c r="N30" s="4" t="inlineStr"/>
+      <c r="O30" s="4" t="inlineStr"/>
+      <c r="P30" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 10:20:00</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>10:20:00</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr"/>
+      <c r="M31" s="4" t="inlineStr"/>
+      <c r="N31" s="4" t="inlineStr"/>
+      <c r="O31" s="4" t="inlineStr"/>
+      <c r="P31" s="4" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>

</xml_diff>

<commit_message>
Implement opening OI cache to fix Change in OI calculation - captures true day opening values
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2038,6 +2038,606 @@
       <c r="N31" s="4" t="inlineStr"/>
       <c r="O31" s="4" t="inlineStr"/>
       <c r="P31" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:00:00</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>11:00:00</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr"/>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr"/>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" s="4" t="inlineStr"/>
+      <c r="L32" s="4" t="inlineStr"/>
+      <c r="M32" s="4" t="inlineStr"/>
+      <c r="N32" s="4" t="inlineStr"/>
+      <c r="O32" s="4" t="inlineStr"/>
+      <c r="P32" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:00:00</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>11:00:00</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" s="4" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr"/>
+      <c r="M33" s="4" t="inlineStr"/>
+      <c r="N33" s="4" t="inlineStr"/>
+      <c r="O33" s="4" t="inlineStr"/>
+      <c r="P33" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:05:00</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>11:05:00</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr"/>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" s="4" t="inlineStr"/>
+      <c r="L34" s="4" t="inlineStr"/>
+      <c r="M34" s="4" t="inlineStr"/>
+      <c r="N34" s="4" t="inlineStr"/>
+      <c r="O34" s="4" t="inlineStr"/>
+      <c r="P34" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:05:00</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>11:05:00</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="4" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr"/>
+      <c r="M35" s="4" t="inlineStr"/>
+      <c r="N35" s="4" t="inlineStr"/>
+      <c r="O35" s="4" t="inlineStr"/>
+      <c r="P35" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:10:00</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>11:10:00</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr"/>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr"/>
+      <c r="K36" s="4" t="inlineStr"/>
+      <c r="L36" s="4" t="inlineStr"/>
+      <c r="M36" s="4" t="inlineStr"/>
+      <c r="N36" s="4" t="inlineStr"/>
+      <c r="O36" s="4" t="inlineStr"/>
+      <c r="P36" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:10:00</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>11:10:00</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr"/>
+      <c r="M37" s="4" t="inlineStr"/>
+      <c r="N37" s="4" t="inlineStr"/>
+      <c r="O37" s="4" t="inlineStr"/>
+      <c r="P37" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:15:00</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>11:15:00</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr"/>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr"/>
+      <c r="K38" s="4" t="inlineStr"/>
+      <c r="L38" s="4" t="inlineStr"/>
+      <c r="M38" s="4" t="inlineStr"/>
+      <c r="N38" s="4" t="inlineStr"/>
+      <c r="O38" s="4" t="inlineStr"/>
+      <c r="P38" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:15:00</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>11:15:00</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr"/>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr"/>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr"/>
+      <c r="M39" s="4" t="inlineStr"/>
+      <c r="N39" s="4" t="inlineStr"/>
+      <c r="O39" s="4" t="inlineStr"/>
+      <c r="P39" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:20:00</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>11:20:00</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr"/>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr"/>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="4" t="inlineStr"/>
+      <c r="M40" s="4" t="inlineStr"/>
+      <c r="N40" s="4" t="inlineStr"/>
+      <c r="O40" s="4" t="inlineStr"/>
+      <c r="P40" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:20:00</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>11:20:00</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr"/>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr"/>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="4" t="inlineStr"/>
+      <c r="M41" s="4" t="inlineStr"/>
+      <c r="N41" s="4" t="inlineStr"/>
+      <c r="O41" s="4" t="inlineStr"/>
+      <c r="P41" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:25:00</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>11:25:00</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr"/>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr"/>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="4" t="inlineStr"/>
+      <c r="M42" s="4" t="inlineStr"/>
+      <c r="N42" s="4" t="inlineStr"/>
+      <c r="O42" s="4" t="inlineStr"/>
+      <c r="P42" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:25:00</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>11:25:00</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr"/>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr"/>
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr"/>
+      <c r="M43" s="4" t="inlineStr"/>
+      <c r="N43" s="4" t="inlineStr"/>
+      <c r="O43" s="4" t="inlineStr"/>
+      <c r="P43" s="4" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>

</xml_diff>

<commit_message>
Update all project files and configuration
- Updated environment configurations
- Updated logging files
- Updated static assets (JS and HTML for open interest chart)
- Cleaned up unnecessary log files
- All changes committed to main branch
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -33,7 +33,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +50,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF70AD47"/>
         <bgColor rgb="FF70AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -101,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -113,6 +125,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -480,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:P87"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2643,6 +2661,2214 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 12:00:00</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>12:00:00</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr"/>
+      <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="4" t="inlineStr"/>
+      <c r="M44" s="4" t="inlineStr"/>
+      <c r="N44" s="4" t="inlineStr"/>
+      <c r="O44" s="4" t="inlineStr"/>
+      <c r="P44" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 12:00:00</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>12:00:00</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr"/>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr"/>
+      <c r="M45" s="4" t="inlineStr"/>
+      <c r="N45" s="4" t="inlineStr"/>
+      <c r="O45" s="4" t="inlineStr"/>
+      <c r="P45" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 12:25:00</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>12:25:00</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr"/>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr"/>
+      <c r="K46" s="4" t="inlineStr"/>
+      <c r="L46" s="4" t="inlineStr"/>
+      <c r="M46" s="4" t="inlineStr"/>
+      <c r="N46" s="4" t="inlineStr"/>
+      <c r="O46" s="4" t="inlineStr"/>
+      <c r="P46" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 12:25:00</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>12:25:00</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr"/>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr"/>
+      <c r="M47" s="4" t="inlineStr"/>
+      <c r="N47" s="4" t="inlineStr"/>
+      <c r="O47" s="4" t="inlineStr"/>
+      <c r="P47" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 13:40:00</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>13:40:00</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr"/>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr"/>
+      <c r="K48" s="4" t="inlineStr"/>
+      <c r="L48" s="4" t="inlineStr"/>
+      <c r="M48" s="4" t="inlineStr"/>
+      <c r="N48" s="4" t="inlineStr"/>
+      <c r="O48" s="4" t="inlineStr"/>
+      <c r="P48" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 13:40:00</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>13:40:00</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr"/>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr"/>
+      <c r="K49" s="4" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr"/>
+      <c r="M49" s="4" t="inlineStr"/>
+      <c r="N49" s="4" t="inlineStr"/>
+      <c r="O49" s="4" t="inlineStr"/>
+      <c r="P49" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 13:45:00</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>13:45:00</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr"/>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr"/>
+      <c r="K50" s="4" t="inlineStr"/>
+      <c r="L50" s="4" t="inlineStr"/>
+      <c r="M50" s="4" t="inlineStr"/>
+      <c r="N50" s="4" t="inlineStr"/>
+      <c r="O50" s="4" t="inlineStr"/>
+      <c r="P50" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 13:45:00</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>13:45:00</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr"/>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr"/>
+      <c r="K51" s="4" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr"/>
+      <c r="M51" s="4" t="inlineStr"/>
+      <c r="N51" s="4" t="inlineStr"/>
+      <c r="O51" s="4" t="inlineStr"/>
+      <c r="P51" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 13:50:00</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>13:50:00</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr"/>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="inlineStr"/>
+      <c r="K52" s="4" t="inlineStr"/>
+      <c r="L52" s="4" t="inlineStr"/>
+      <c r="M52" s="4" t="inlineStr"/>
+      <c r="N52" s="4" t="inlineStr"/>
+      <c r="O52" s="4" t="inlineStr"/>
+      <c r="P52" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 13:50:00</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>13:50:00</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr"/>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="inlineStr"/>
+      <c r="K53" s="4" t="inlineStr"/>
+      <c r="L53" s="4" t="inlineStr"/>
+      <c r="M53" s="4" t="inlineStr"/>
+      <c r="N53" s="4" t="inlineStr"/>
+      <c r="O53" s="4" t="inlineStr"/>
+      <c r="P53" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 13:55:00</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>13:55:00</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr"/>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr"/>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr"/>
+      <c r="K54" s="4" t="inlineStr"/>
+      <c r="L54" s="4" t="inlineStr"/>
+      <c r="M54" s="4" t="inlineStr"/>
+      <c r="N54" s="4" t="inlineStr"/>
+      <c r="O54" s="4" t="inlineStr"/>
+      <c r="P54" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 13:55:00</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>13:55:00</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr"/>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr"/>
+      <c r="K55" s="4" t="inlineStr"/>
+      <c r="L55" s="4" t="inlineStr"/>
+      <c r="M55" s="4" t="inlineStr"/>
+      <c r="N55" s="4" t="inlineStr"/>
+      <c r="O55" s="4" t="inlineStr"/>
+      <c r="P55" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:00:00</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr"/>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr"/>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr"/>
+      <c r="K56" s="4" t="inlineStr"/>
+      <c r="L56" s="4" t="inlineStr"/>
+      <c r="M56" s="4" t="inlineStr"/>
+      <c r="N56" s="4" t="inlineStr"/>
+      <c r="O56" s="4" t="inlineStr"/>
+      <c r="P56" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:00:00</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr"/>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr"/>
+      <c r="K57" s="4" t="inlineStr"/>
+      <c r="L57" s="4" t="inlineStr"/>
+      <c r="M57" s="4" t="inlineStr"/>
+      <c r="N57" s="4" t="inlineStr"/>
+      <c r="O57" s="4" t="inlineStr"/>
+      <c r="P57" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:05:00</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>14:05:00</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr"/>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr"/>
+      <c r="K58" s="4" t="inlineStr"/>
+      <c r="L58" s="4" t="inlineStr"/>
+      <c r="M58" s="4" t="inlineStr"/>
+      <c r="N58" s="4" t="inlineStr"/>
+      <c r="O58" s="4" t="inlineStr"/>
+      <c r="P58" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:05:00</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>14:05:00</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr"/>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr"/>
+      <c r="K59" s="4" t="inlineStr"/>
+      <c r="L59" s="4" t="inlineStr"/>
+      <c r="M59" s="4" t="inlineStr"/>
+      <c r="N59" s="4" t="inlineStr"/>
+      <c r="O59" s="4" t="inlineStr"/>
+      <c r="P59" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:10:00</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>14:10:00</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr"/>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr"/>
+      <c r="K60" s="4" t="inlineStr"/>
+      <c r="L60" s="4" t="inlineStr"/>
+      <c r="M60" s="4" t="inlineStr"/>
+      <c r="N60" s="4" t="inlineStr"/>
+      <c r="O60" s="4" t="inlineStr"/>
+      <c r="P60" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:10:00</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>14:10:00</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr"/>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr"/>
+      <c r="K61" s="4" t="inlineStr"/>
+      <c r="L61" s="4" t="inlineStr"/>
+      <c r="M61" s="4" t="inlineStr"/>
+      <c r="N61" s="4" t="inlineStr"/>
+      <c r="O61" s="4" t="inlineStr"/>
+      <c r="P61" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:15:00</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>14:15:00</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr"/>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr"/>
+      <c r="K62" s="4" t="inlineStr"/>
+      <c r="L62" s="4" t="inlineStr"/>
+      <c r="M62" s="4" t="inlineStr"/>
+      <c r="N62" s="4" t="inlineStr"/>
+      <c r="O62" s="4" t="inlineStr"/>
+      <c r="P62" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:15:00</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>14:15:00</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr"/>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr"/>
+      <c r="K63" s="4" t="inlineStr"/>
+      <c r="L63" s="4" t="inlineStr"/>
+      <c r="M63" s="4" t="inlineStr"/>
+      <c r="N63" s="4" t="inlineStr"/>
+      <c r="O63" s="4" t="inlineStr"/>
+      <c r="P63" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:20:00</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>14:20:00</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr"/>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr"/>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr"/>
+      <c r="K64" s="4" t="inlineStr"/>
+      <c r="L64" s="4" t="inlineStr"/>
+      <c r="M64" s="4" t="inlineStr"/>
+      <c r="N64" s="4" t="inlineStr"/>
+      <c r="O64" s="4" t="inlineStr"/>
+      <c r="P64" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:20:00</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>14:20:00</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr"/>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="inlineStr"/>
+      <c r="K65" s="4" t="inlineStr"/>
+      <c r="L65" s="4" t="inlineStr"/>
+      <c r="M65" s="4" t="inlineStr"/>
+      <c r="N65" s="4" t="inlineStr"/>
+      <c r="O65" s="4" t="inlineStr"/>
+      <c r="P65" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:25:00</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>14:25:00</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr"/>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr"/>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="inlineStr"/>
+      <c r="K66" s="4" t="inlineStr"/>
+      <c r="L66" s="4" t="inlineStr"/>
+      <c r="M66" s="4" t="inlineStr"/>
+      <c r="N66" s="4" t="inlineStr"/>
+      <c r="O66" s="4" t="inlineStr"/>
+      <c r="P66" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:25:00</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>14:25:00</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr"/>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr"/>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr"/>
+      <c r="K67" s="4" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr"/>
+      <c r="M67" s="4" t="inlineStr"/>
+      <c r="N67" s="4" t="inlineStr"/>
+      <c r="O67" s="4" t="inlineStr"/>
+      <c r="P67" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:30:00</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>14:30:00</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr"/>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr"/>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr"/>
+      <c r="K68" s="4" t="inlineStr"/>
+      <c r="L68" s="4" t="inlineStr"/>
+      <c r="M68" s="4" t="inlineStr"/>
+      <c r="N68" s="4" t="inlineStr"/>
+      <c r="O68" s="4" t="inlineStr"/>
+      <c r="P68" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:30:00</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>14:30:00</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr"/>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr"/>
+      <c r="K69" s="4" t="inlineStr"/>
+      <c r="L69" s="4" t="inlineStr"/>
+      <c r="M69" s="4" t="inlineStr"/>
+      <c r="N69" s="4" t="inlineStr"/>
+      <c r="O69" s="4" t="inlineStr"/>
+      <c r="P69" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:35:00</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>14:35:00</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr"/>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr"/>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr"/>
+      <c r="K70" s="4" t="inlineStr"/>
+      <c r="L70" s="4" t="inlineStr"/>
+      <c r="M70" s="4" t="inlineStr"/>
+      <c r="N70" s="4" t="inlineStr"/>
+      <c r="O70" s="4" t="inlineStr"/>
+      <c r="P70" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:35:00</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>14:35:00</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr"/>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr"/>
+      <c r="K71" s="4" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr"/>
+      <c r="M71" s="4" t="inlineStr"/>
+      <c r="N71" s="4" t="inlineStr"/>
+      <c r="O71" s="4" t="inlineStr"/>
+      <c r="P71" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:40:00</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>14:40:00</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr"/>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr"/>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr"/>
+      <c r="K72" s="4" t="inlineStr"/>
+      <c r="L72" s="4" t="inlineStr"/>
+      <c r="M72" s="4" t="inlineStr"/>
+      <c r="N72" s="4" t="inlineStr"/>
+      <c r="O72" s="4" t="inlineStr"/>
+      <c r="P72" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:40:00</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>14:40:00</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr"/>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr"/>
+      <c r="K73" s="4" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr"/>
+      <c r="M73" s="4" t="inlineStr"/>
+      <c r="N73" s="4" t="inlineStr"/>
+      <c r="O73" s="4" t="inlineStr"/>
+      <c r="P73" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:45:00</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr"/>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr"/>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr"/>
+      <c r="K74" s="4" t="inlineStr"/>
+      <c r="L74" s="4" t="inlineStr"/>
+      <c r="M74" s="4" t="inlineStr"/>
+      <c r="N74" s="4" t="inlineStr"/>
+      <c r="O74" s="4" t="inlineStr"/>
+      <c r="P74" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:45:00</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr"/>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr"/>
+      <c r="K75" s="4" t="inlineStr"/>
+      <c r="L75" s="4" t="inlineStr"/>
+      <c r="M75" s="4" t="inlineStr"/>
+      <c r="N75" s="4" t="inlineStr"/>
+      <c r="O75" s="4" t="inlineStr"/>
+      <c r="P75" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:50:00</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr"/>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr"/>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr">
+        <is>
+          <t>✓ YES</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr"/>
+      <c r="K76" s="4" t="inlineStr">
+        <is>
+          <t>173.55</t>
+        </is>
+      </c>
+      <c r="L76" s="4" t="inlineStr"/>
+      <c r="M76" s="4" t="inlineStr">
+        <is>
+          <t>146.60</t>
+        </is>
+      </c>
+      <c r="N76" s="4" t="inlineStr"/>
+      <c r="O76" s="4" t="inlineStr">
+        <is>
+          <t>227.45</t>
+        </is>
+      </c>
+      <c r="P76" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:50:00</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr"/>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr"/>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr">
+        <is>
+          <t>✓ YES</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr"/>
+      <c r="K77" s="4" t="inlineStr">
+        <is>
+          <t>173.55</t>
+        </is>
+      </c>
+      <c r="L77" s="4" t="inlineStr"/>
+      <c r="M77" s="4" t="inlineStr">
+        <is>
+          <t>146.60</t>
+        </is>
+      </c>
+      <c r="N77" s="4" t="inlineStr"/>
+      <c r="O77" s="4" t="inlineStr">
+        <is>
+          <t>227.45</t>
+        </is>
+      </c>
+      <c r="P77" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:55:00</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>14:55:00</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr"/>
+      <c r="E78" s="4" t="inlineStr"/>
+      <c r="F78" s="4" t="inlineStr"/>
+      <c r="G78" s="4" t="inlineStr"/>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr"/>
+      <c r="K78" s="4" t="inlineStr"/>
+      <c r="L78" s="4" t="inlineStr"/>
+      <c r="M78" s="4" t="inlineStr"/>
+      <c r="N78" s="4" t="inlineStr"/>
+      <c r="O78" s="4" t="inlineStr"/>
+      <c r="P78" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Live data fetch timed out after 45s - candle fetching took too long, retrying next cycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:55:00</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>14:55:00</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr"/>
+      <c r="E79" s="4" t="inlineStr"/>
+      <c r="F79" s="4" t="inlineStr"/>
+      <c r="G79" s="4" t="inlineStr"/>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr"/>
+      <c r="K79" s="4" t="inlineStr"/>
+      <c r="L79" s="4" t="inlineStr"/>
+      <c r="M79" s="4" t="inlineStr"/>
+      <c r="N79" s="4" t="inlineStr"/>
+      <c r="O79" s="4" t="inlineStr"/>
+      <c r="P79" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Live data fetch timed out after 45s - candle fetching took too long, retrying next cycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 15:00:00</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr"/>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr"/>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr"/>
+      <c r="K80" s="4" t="inlineStr"/>
+      <c r="L80" s="4" t="inlineStr"/>
+      <c r="M80" s="4" t="inlineStr"/>
+      <c r="N80" s="4" t="inlineStr"/>
+      <c r="O80" s="4" t="inlineStr"/>
+      <c r="P80" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 15:00:00</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr"/>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr"/>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr"/>
+      <c r="K81" s="4" t="inlineStr"/>
+      <c r="L81" s="4" t="inlineStr"/>
+      <c r="M81" s="4" t="inlineStr"/>
+      <c r="N81" s="4" t="inlineStr"/>
+      <c r="O81" s="4" t="inlineStr"/>
+      <c r="P81" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 15:05:00</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>15:05:00</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr"/>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr"/>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr"/>
+      <c r="K82" s="4" t="inlineStr"/>
+      <c r="L82" s="4" t="inlineStr"/>
+      <c r="M82" s="4" t="inlineStr"/>
+      <c r="N82" s="4" t="inlineStr"/>
+      <c r="O82" s="4" t="inlineStr"/>
+      <c r="P82" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 15:05:00</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>15:05:00</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr"/>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr"/>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr"/>
+      <c r="K83" s="4" t="inlineStr"/>
+      <c r="L83" s="4" t="inlineStr"/>
+      <c r="M83" s="4" t="inlineStr"/>
+      <c r="N83" s="4" t="inlineStr"/>
+      <c r="O83" s="4" t="inlineStr"/>
+      <c r="P83" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 15:10:00</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>15:10:00</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr"/>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr"/>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr"/>
+      <c r="K84" s="4" t="inlineStr"/>
+      <c r="L84" s="4" t="inlineStr"/>
+      <c r="M84" s="4" t="inlineStr"/>
+      <c r="N84" s="4" t="inlineStr"/>
+      <c r="O84" s="4" t="inlineStr"/>
+      <c r="P84" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 15:10:00</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>15:10:00</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr"/>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr"/>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr"/>
+      <c r="K85" s="4" t="inlineStr"/>
+      <c r="L85" s="4" t="inlineStr"/>
+      <c r="M85" s="4" t="inlineStr"/>
+      <c r="N85" s="4" t="inlineStr"/>
+      <c r="O85" s="4" t="inlineStr"/>
+      <c r="P85" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 15:15:00</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>15:15:00</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>156.60</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr"/>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>124.55</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr"/>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr"/>
+      <c r="K86" s="4" t="inlineStr"/>
+      <c r="L86" s="4" t="inlineStr"/>
+      <c r="M86" s="4" t="inlineStr"/>
+      <c r="N86" s="4" t="inlineStr"/>
+      <c r="O86" s="4" t="inlineStr"/>
+      <c r="P86" s="4" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 15:15:00</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>15:15:00</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>169.80</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr"/>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>101.15</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr"/>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr"/>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
+      <c r="M87" s="4" t="inlineStr"/>
+      <c r="N87" s="4" t="inlineStr"/>
+      <c r="O87" s="4" t="inlineStr"/>
+      <c r="P87" s="4" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2654,7 +4880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2729,6 +4955,106 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:50:05</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>BUY PE</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>25900</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>173.55</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>173.55</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr"/>
+      <c r="I2" s="4" t="inlineStr"/>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>BUY PE</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>2021876953262776320</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Mode: LIVE | Details: Order placed successfully via KiteService | Order_type: MARKET</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2026-02-12 14:50:05</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>SL_ORDER</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>25900</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>146.60</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>227.45</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>146.60</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>PLACED</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>2021876953866756096</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>SL Order Placed | Trigger: 146.60</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: remove unused python scripts and verification files
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -579,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P84"/>
+  <dimension ref="A1:P90"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4763,6 +4763,306 @@
       <c r="N84" s="10" t="inlineStr"/>
       <c r="O84" s="10" t="inlineStr"/>
       <c r="P84" s="10" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-17 12:50:00</t>
+        </is>
+      </c>
+      <c r="B85" s="10" t="inlineStr">
+        <is>
+          <t>12:50:00</t>
+        </is>
+      </c>
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="D85" s="10" t="inlineStr">
+        <is>
+          <t>85.00</t>
+        </is>
+      </c>
+      <c r="E85" s="10" t="inlineStr"/>
+      <c r="F85" s="10" t="inlineStr">
+        <is>
+          <t>128.55</t>
+        </is>
+      </c>
+      <c r="G85" s="10" t="inlineStr"/>
+      <c r="H85" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I85" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J85" s="10" t="inlineStr"/>
+      <c r="K85" s="10" t="inlineStr"/>
+      <c r="L85" s="10" t="inlineStr"/>
+      <c r="M85" s="10" t="inlineStr"/>
+      <c r="N85" s="10" t="inlineStr"/>
+      <c r="O85" s="10" t="inlineStr"/>
+      <c r="P85" s="10" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-17 12:50:00</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t>12:50:00</t>
+        </is>
+      </c>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="D86" s="10" t="inlineStr">
+        <is>
+          <t>118.00</t>
+        </is>
+      </c>
+      <c r="E86" s="10" t="inlineStr"/>
+      <c r="F86" s="10" t="inlineStr">
+        <is>
+          <t>65.00</t>
+        </is>
+      </c>
+      <c r="G86" s="10" t="inlineStr"/>
+      <c r="H86" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I86" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J86" s="10" t="inlineStr"/>
+      <c r="K86" s="10" t="inlineStr"/>
+      <c r="L86" s="10" t="inlineStr"/>
+      <c r="M86" s="10" t="inlineStr"/>
+      <c r="N86" s="10" t="inlineStr"/>
+      <c r="O86" s="10" t="inlineStr"/>
+      <c r="P86" s="10" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-17 14:00:00</t>
+        </is>
+      </c>
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="C87" s="10" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D87" s="10" t="inlineStr">
+        <is>
+          <t>85.00</t>
+        </is>
+      </c>
+      <c r="E87" s="10" t="inlineStr"/>
+      <c r="F87" s="10" t="inlineStr">
+        <is>
+          <t>128.55</t>
+        </is>
+      </c>
+      <c r="G87" s="10" t="inlineStr"/>
+      <c r="H87" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I87" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J87" s="10" t="inlineStr"/>
+      <c r="K87" s="10" t="inlineStr"/>
+      <c r="L87" s="10" t="inlineStr"/>
+      <c r="M87" s="10" t="inlineStr"/>
+      <c r="N87" s="10" t="inlineStr"/>
+      <c r="O87" s="10" t="inlineStr"/>
+      <c r="P87" s="10" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-17 14:00:00</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D88" s="10" t="inlineStr">
+        <is>
+          <t>118.00</t>
+        </is>
+      </c>
+      <c r="E88" s="10" t="inlineStr"/>
+      <c r="F88" s="10" t="inlineStr">
+        <is>
+          <t>65.00</t>
+        </is>
+      </c>
+      <c r="G88" s="10" t="inlineStr"/>
+      <c r="H88" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I88" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J88" s="10" t="inlineStr"/>
+      <c r="K88" s="10" t="inlineStr"/>
+      <c r="L88" s="10" t="inlineStr"/>
+      <c r="M88" s="10" t="inlineStr"/>
+      <c r="N88" s="10" t="inlineStr"/>
+      <c r="O88" s="10" t="inlineStr"/>
+      <c r="P88" s="10" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-17 14:05:00</t>
+        </is>
+      </c>
+      <c r="B89" s="10" t="inlineStr">
+        <is>
+          <t>14:05:00</t>
+        </is>
+      </c>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="D89" s="10" t="inlineStr">
+        <is>
+          <t>85.00</t>
+        </is>
+      </c>
+      <c r="E89" s="10" t="inlineStr"/>
+      <c r="F89" s="10" t="inlineStr">
+        <is>
+          <t>128.55</t>
+        </is>
+      </c>
+      <c r="G89" s="10" t="inlineStr"/>
+      <c r="H89" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I89" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J89" s="10" t="inlineStr"/>
+      <c r="K89" s="10" t="inlineStr"/>
+      <c r="L89" s="10" t="inlineStr"/>
+      <c r="M89" s="10" t="inlineStr"/>
+      <c r="N89" s="10" t="inlineStr"/>
+      <c r="O89" s="10" t="inlineStr"/>
+      <c r="P89" s="10" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-17 14:05:00</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t>14:05:00</t>
+        </is>
+      </c>
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="D90" s="10" t="inlineStr">
+        <is>
+          <t>118.00</t>
+        </is>
+      </c>
+      <c r="E90" s="10" t="inlineStr"/>
+      <c r="F90" s="10" t="inlineStr">
+        <is>
+          <t>65.00</t>
+        </is>
+      </c>
+      <c r="G90" s="10" t="inlineStr"/>
+      <c r="H90" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I90" s="10" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J90" s="10" t="inlineStr"/>
+      <c r="K90" s="10" t="inlineStr"/>
+      <c r="L90" s="10" t="inlineStr"/>
+      <c r="M90" s="10" t="inlineStr"/>
+      <c r="N90" s="10" t="inlineStr"/>
+      <c r="O90" s="10" t="inlineStr"/>
+      <c r="P90" s="10" t="inlineStr">
         <is>
           <t>Low Strike Check</t>
         </is>

</xml_diff>

<commit_message>
Update signal logs and live signal script
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,8 +32,12 @@
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -98,6 +102,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+        <bgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -224,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -275,6 +285,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -642,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P128"/>
+  <dimension ref="A1:P137"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6951,6 +6965,388 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" s="15" t="inlineStr">
+        <is>
+          <t>2026-02-21 11:30:00</t>
+        </is>
+      </c>
+      <c r="B129" s="15" t="inlineStr">
+        <is>
+          <t>11:30:00</t>
+        </is>
+      </c>
+      <c r="C129" s="15" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D129" s="15" t="inlineStr"/>
+      <c r="E129" s="15" t="inlineStr"/>
+      <c r="F129" s="15" t="inlineStr"/>
+      <c r="G129" s="15" t="inlineStr"/>
+      <c r="H129" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I129" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J129" s="15" t="inlineStr"/>
+      <c r="K129" s="15" t="inlineStr"/>
+      <c r="L129" s="15" t="inlineStr"/>
+      <c r="M129" s="15" t="inlineStr"/>
+      <c r="N129" s="15" t="inlineStr"/>
+      <c r="O129" s="15" t="inlineStr"/>
+      <c r="P129" s="15" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="15" t="inlineStr">
+        <is>
+          <t>2026-02-21 11:30:00</t>
+        </is>
+      </c>
+      <c r="B130" s="15" t="inlineStr">
+        <is>
+          <t>11:30:00</t>
+        </is>
+      </c>
+      <c r="C130" s="15" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D130" s="15" t="inlineStr"/>
+      <c r="E130" s="15" t="inlineStr"/>
+      <c r="F130" s="15" t="inlineStr"/>
+      <c r="G130" s="15" t="inlineStr"/>
+      <c r="H130" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I130" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J130" s="15" t="inlineStr"/>
+      <c r="K130" s="15" t="inlineStr"/>
+      <c r="L130" s="15" t="inlineStr"/>
+      <c r="M130" s="15" t="inlineStr"/>
+      <c r="N130" s="15" t="inlineStr"/>
+      <c r="O130" s="15" t="inlineStr"/>
+      <c r="P130" s="15" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="15" t="inlineStr">
+        <is>
+          <t>2026-02-21 11:45:00</t>
+        </is>
+      </c>
+      <c r="B131" s="15" t="inlineStr">
+        <is>
+          <t>11:45:00</t>
+        </is>
+      </c>
+      <c r="C131" s="15" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D131" s="15" t="inlineStr"/>
+      <c r="E131" s="15" t="inlineStr"/>
+      <c r="F131" s="15" t="inlineStr"/>
+      <c r="G131" s="15" t="inlineStr"/>
+      <c r="H131" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I131" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J131" s="15" t="inlineStr"/>
+      <c r="K131" s="15" t="inlineStr"/>
+      <c r="L131" s="15" t="inlineStr"/>
+      <c r="M131" s="15" t="inlineStr"/>
+      <c r="N131" s="15" t="inlineStr"/>
+      <c r="O131" s="15" t="inlineStr"/>
+      <c r="P131" s="15" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="15" t="inlineStr">
+        <is>
+          <t>2026-02-21 11:45:00</t>
+        </is>
+      </c>
+      <c r="B132" s="15" t="inlineStr">
+        <is>
+          <t>11:45:00</t>
+        </is>
+      </c>
+      <c r="C132" s="15" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D132" s="15" t="inlineStr"/>
+      <c r="E132" s="15" t="inlineStr"/>
+      <c r="F132" s="15" t="inlineStr"/>
+      <c r="G132" s="15" t="inlineStr"/>
+      <c r="H132" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I132" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J132" s="15" t="inlineStr"/>
+      <c r="K132" s="15" t="inlineStr"/>
+      <c r="L132" s="15" t="inlineStr"/>
+      <c r="M132" s="15" t="inlineStr"/>
+      <c r="N132" s="15" t="inlineStr"/>
+      <c r="O132" s="15" t="inlineStr"/>
+      <c r="P132" s="15" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="15" t="inlineStr">
+        <is>
+          <t>2026-02-21 13:00:00</t>
+        </is>
+      </c>
+      <c r="B133" s="15" t="inlineStr">
+        <is>
+          <t>13:00:00</t>
+        </is>
+      </c>
+      <c r="C133" s="15" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D133" s="15" t="inlineStr"/>
+      <c r="E133" s="15" t="inlineStr"/>
+      <c r="F133" s="15" t="inlineStr"/>
+      <c r="G133" s="15" t="inlineStr"/>
+      <c r="H133" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I133" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J133" s="15" t="inlineStr"/>
+      <c r="K133" s="15" t="inlineStr"/>
+      <c r="L133" s="15" t="inlineStr"/>
+      <c r="M133" s="15" t="inlineStr"/>
+      <c r="N133" s="15" t="inlineStr"/>
+      <c r="O133" s="15" t="inlineStr"/>
+      <c r="P133" s="15" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="15" t="inlineStr">
+        <is>
+          <t>2026-02-21 13:00:00</t>
+        </is>
+      </c>
+      <c r="B134" s="15" t="inlineStr">
+        <is>
+          <t>13:00:00</t>
+        </is>
+      </c>
+      <c r="C134" s="15" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D134" s="15" t="inlineStr"/>
+      <c r="E134" s="15" t="inlineStr"/>
+      <c r="F134" s="15" t="inlineStr"/>
+      <c r="G134" s="15" t="inlineStr"/>
+      <c r="H134" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I134" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J134" s="15" t="inlineStr"/>
+      <c r="K134" s="15" t="inlineStr"/>
+      <c r="L134" s="15" t="inlineStr"/>
+      <c r="M134" s="15" t="inlineStr"/>
+      <c r="N134" s="15" t="inlineStr"/>
+      <c r="O134" s="15" t="inlineStr"/>
+      <c r="P134" s="15" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="18" t="inlineStr">
+        <is>
+          <t>2026-02-21 15:33:58</t>
+        </is>
+      </c>
+      <c r="B135" s="18" t="inlineStr">
+        <is>
+          <t>15:33:58</t>
+        </is>
+      </c>
+      <c r="C135" s="18" t="inlineStr">
+        <is>
+          <t>15:33</t>
+        </is>
+      </c>
+      <c r="D135" s="19" t="n">
+        <v>25450</v>
+      </c>
+      <c r="E135" s="19" t="inlineStr"/>
+      <c r="F135" s="19" t="inlineStr"/>
+      <c r="G135" s="19" t="inlineStr"/>
+      <c r="H135" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I135" s="19" t="inlineStr"/>
+      <c r="J135" s="19" t="n">
+        <v>207.1</v>
+      </c>
+      <c r="K135" s="19" t="inlineStr"/>
+      <c r="L135" s="19" t="n">
+        <v>180.8</v>
+      </c>
+      <c r="M135" s="19" t="inlineStr"/>
+      <c r="N135" s="19" t="n">
+        <v>259.7</v>
+      </c>
+      <c r="O135" s="19" t="inlineStr"/>
+      <c r="P135" s="18" t="inlineStr">
+        <is>
+          <t>CE MARKET_CLOSE | Strike: 25450 | Price: 207.10 | Entry: 207.10 | SL: 180.80 | Target: 259.70 | PnL: +0.00 (+0.00%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="15" t="inlineStr">
+        <is>
+          <t>2026-02-21 14:50:00</t>
+        </is>
+      </c>
+      <c r="B136" s="15" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C136" s="15" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D136" s="15" t="inlineStr"/>
+      <c r="E136" s="15" t="inlineStr"/>
+      <c r="F136" s="15" t="inlineStr"/>
+      <c r="G136" s="15" t="inlineStr"/>
+      <c r="H136" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I136" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J136" s="15" t="inlineStr"/>
+      <c r="K136" s="15" t="inlineStr"/>
+      <c r="L136" s="15" t="inlineStr"/>
+      <c r="M136" s="15" t="inlineStr"/>
+      <c r="N136" s="15" t="inlineStr"/>
+      <c r="O136" s="15" t="inlineStr"/>
+      <c r="P136" s="15" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="15" t="inlineStr">
+        <is>
+          <t>2026-02-21 14:50:00</t>
+        </is>
+      </c>
+      <c r="B137" s="15" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C137" s="15" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D137" s="15" t="inlineStr"/>
+      <c r="E137" s="15" t="inlineStr"/>
+      <c r="F137" s="15" t="inlineStr"/>
+      <c r="G137" s="15" t="inlineStr"/>
+      <c r="H137" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I137" s="15" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J137" s="15" t="inlineStr"/>
+      <c r="K137" s="15" t="inlineStr"/>
+      <c r="L137" s="15" t="inlineStr"/>
+      <c r="M137" s="15" t="inlineStr"/>
+      <c r="N137" s="15" t="inlineStr"/>
+      <c r="O137" s="15" t="inlineStr"/>
+      <c r="P137" s="15" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6962,7 +7358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8037,6 +8433,106 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>2026-02-21 15:34:01</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>SELL CE</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>25450</v>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>207.10</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>207.10</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr"/>
+      <c r="H22" s="15" t="inlineStr"/>
+      <c r="I22" s="15" t="inlineStr"/>
+      <c r="J22" s="16" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="K22" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L22" s="15" t="inlineStr">
+        <is>
+          <t>Mode: LIVE | Error: Incorrect `api_key` or `access_token`. | Details: Exit Reason: Market Close (3:20 PM) | Order_type: MARKET</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>2026-02-21 15:34:01</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>25450</v>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>207.10</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>207.10</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>259.70</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>180.80</t>
+        </is>
+      </c>
+      <c r="I23" s="15" t="inlineStr"/>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>MARKET_CLOSE</t>
+        </is>
+      </c>
+      <c r="K23" s="15" t="inlineStr"/>
+      <c r="L23" s="15" t="inlineStr">
+        <is>
+          <t>Market Close Square-Off (3:20 PM) | Entry Time: 2026-02-20T13:15:08.706661 | Entry Order ID: 2024752161975885824 | Entry Price: 207.10 | Stop Loss: 180.8 | Exit Price: 207.10 | P&amp;L: +0.00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Catch Kotak Neo API 'View Token' 401 error and correctly ask user to update KOTAK_ACCESS_TOKEN
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -814,6 +814,390 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-25 09:20:00</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>09:20:00</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>185.45</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>200.00</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr"/>
+      <c r="N7" s="3" t="inlineStr"/>
+      <c r="O7" s="3" t="inlineStr"/>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-25 09:20:00</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>09:20:00</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>215.50</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>159.00</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr"/>
+      <c r="M8" s="3" t="inlineStr"/>
+      <c r="N8" s="3" t="inlineStr"/>
+      <c r="O8" s="3" t="inlineStr"/>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-25 09:25:00</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>09:25:00</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>09:25</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>185.45</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>200.00</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr"/>
+      <c r="N9" s="3" t="inlineStr"/>
+      <c r="O9" s="3" t="inlineStr"/>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-25 09:25:00</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>09:25:00</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>09:25</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>215.50</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>159.00</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr"/>
+      <c r="N10" s="3" t="inlineStr"/>
+      <c r="O10" s="3" t="inlineStr"/>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-25 09:30:00</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr"/>
+      <c r="M11" s="3" t="inlineStr"/>
+      <c r="N11" s="3" t="inlineStr"/>
+      <c r="O11" s="3" t="inlineStr"/>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Live data fetch timed out after 45s - candle fetching took too long, retrying next cycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-25 09:30:00</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr"/>
+      <c r="M12" s="3" t="inlineStr"/>
+      <c r="N12" s="3" t="inlineStr"/>
+      <c r="O12" s="3" t="inlineStr"/>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Live data fetch timed out after 45s - candle fetching took too long, retrying next cycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-25 09:35:00</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>09:35:00</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>185.45</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>200.00</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr"/>
+      <c r="M13" s="3" t="inlineStr"/>
+      <c r="N13" s="3" t="inlineStr"/>
+      <c r="O13" s="3" t="inlineStr"/>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>High Strike Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-25 09:35:00</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>09:35:00</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>215.50</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>159.00</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr"/>
+      <c r="N14" s="3" t="inlineStr"/>
+      <c r="O14" s="3" t="inlineStr"/>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>Low Strike Check</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add fixed Oracle Cloud deployment script
- oracle_cloud_deploy_fixed.sh: Simplified and robust deployment script
  * Fixes syntax errors from original script
  * 8-phase setup process
  * System updates, Python venv, Gunicorn, Nginx, Firewall, Log rotation
  * Clear step-by-step next steps for application deployment
  * All inline configuration without external file issues

Tested and ready for Oracle Cloud Always Free Tier deployment
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P193"/>
+  <dimension ref="A1:P201"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9888,6 +9888,342 @@
       <c r="N193" s="4" t="inlineStr"/>
       <c r="O193" s="4" t="inlineStr"/>
       <c r="P193" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:25:00</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>11:25:00</t>
+        </is>
+      </c>
+      <c r="C194" s="4" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="D194" s="4" t="inlineStr"/>
+      <c r="E194" s="4" t="inlineStr"/>
+      <c r="F194" s="4" t="inlineStr"/>
+      <c r="G194" s="4" t="inlineStr"/>
+      <c r="H194" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I194" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J194" s="4" t="inlineStr"/>
+      <c r="K194" s="4" t="inlineStr"/>
+      <c r="L194" s="4" t="inlineStr"/>
+      <c r="M194" s="4" t="inlineStr"/>
+      <c r="N194" s="4" t="inlineStr"/>
+      <c r="O194" s="4" t="inlineStr"/>
+      <c r="P194" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:25:00</t>
+        </is>
+      </c>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t>11:25:00</t>
+        </is>
+      </c>
+      <c r="C195" s="4" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="D195" s="4" t="inlineStr"/>
+      <c r="E195" s="4" t="inlineStr"/>
+      <c r="F195" s="4" t="inlineStr"/>
+      <c r="G195" s="4" t="inlineStr"/>
+      <c r="H195" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I195" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J195" s="4" t="inlineStr"/>
+      <c r="K195" s="4" t="inlineStr"/>
+      <c r="L195" s="4" t="inlineStr"/>
+      <c r="M195" s="4" t="inlineStr"/>
+      <c r="N195" s="4" t="inlineStr"/>
+      <c r="O195" s="4" t="inlineStr"/>
+      <c r="P195" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:30:00</t>
+        </is>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>11:30:00</t>
+        </is>
+      </c>
+      <c r="C196" s="4" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D196" s="4" t="inlineStr"/>
+      <c r="E196" s="4" t="inlineStr"/>
+      <c r="F196" s="4" t="inlineStr"/>
+      <c r="G196" s="4" t="inlineStr"/>
+      <c r="H196" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I196" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J196" s="4" t="inlineStr"/>
+      <c r="K196" s="4" t="inlineStr"/>
+      <c r="L196" s="4" t="inlineStr"/>
+      <c r="M196" s="4" t="inlineStr"/>
+      <c r="N196" s="4" t="inlineStr"/>
+      <c r="O196" s="4" t="inlineStr"/>
+      <c r="P196" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:30:00</t>
+        </is>
+      </c>
+      <c r="B197" s="4" t="inlineStr">
+        <is>
+          <t>11:30:00</t>
+        </is>
+      </c>
+      <c r="C197" s="4" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D197" s="4" t="inlineStr"/>
+      <c r="E197" s="4" t="inlineStr"/>
+      <c r="F197" s="4" t="inlineStr"/>
+      <c r="G197" s="4" t="inlineStr"/>
+      <c r="H197" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I197" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J197" s="4" t="inlineStr"/>
+      <c r="K197" s="4" t="inlineStr"/>
+      <c r="L197" s="4" t="inlineStr"/>
+      <c r="M197" s="4" t="inlineStr"/>
+      <c r="N197" s="4" t="inlineStr"/>
+      <c r="O197" s="4" t="inlineStr"/>
+      <c r="P197" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:35:00</t>
+        </is>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>11:35:00</t>
+        </is>
+      </c>
+      <c r="C198" s="4" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="D198" s="4" t="inlineStr"/>
+      <c r="E198" s="4" t="inlineStr"/>
+      <c r="F198" s="4" t="inlineStr"/>
+      <c r="G198" s="4" t="inlineStr"/>
+      <c r="H198" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I198" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J198" s="4" t="inlineStr"/>
+      <c r="K198" s="4" t="inlineStr"/>
+      <c r="L198" s="4" t="inlineStr"/>
+      <c r="M198" s="4" t="inlineStr"/>
+      <c r="N198" s="4" t="inlineStr"/>
+      <c r="O198" s="4" t="inlineStr"/>
+      <c r="P198" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:35:00</t>
+        </is>
+      </c>
+      <c r="B199" s="4" t="inlineStr">
+        <is>
+          <t>11:35:00</t>
+        </is>
+      </c>
+      <c r="C199" s="4" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="D199" s="4" t="inlineStr"/>
+      <c r="E199" s="4" t="inlineStr"/>
+      <c r="F199" s="4" t="inlineStr"/>
+      <c r="G199" s="4" t="inlineStr"/>
+      <c r="H199" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I199" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J199" s="4" t="inlineStr"/>
+      <c r="K199" s="4" t="inlineStr"/>
+      <c r="L199" s="4" t="inlineStr"/>
+      <c r="M199" s="4" t="inlineStr"/>
+      <c r="N199" s="4" t="inlineStr"/>
+      <c r="O199" s="4" t="inlineStr"/>
+      <c r="P199" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:40:00</t>
+        </is>
+      </c>
+      <c r="B200" s="4" t="inlineStr">
+        <is>
+          <t>11:40:00</t>
+        </is>
+      </c>
+      <c r="C200" s="4" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="D200" s="4" t="inlineStr"/>
+      <c r="E200" s="4" t="inlineStr"/>
+      <c r="F200" s="4" t="inlineStr"/>
+      <c r="G200" s="4" t="inlineStr"/>
+      <c r="H200" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I200" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J200" s="4" t="inlineStr"/>
+      <c r="K200" s="4" t="inlineStr"/>
+      <c r="L200" s="4" t="inlineStr"/>
+      <c r="M200" s="4" t="inlineStr"/>
+      <c r="N200" s="4" t="inlineStr"/>
+      <c r="O200" s="4" t="inlineStr"/>
+      <c r="P200" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:40:00</t>
+        </is>
+      </c>
+      <c r="B201" s="4" t="inlineStr">
+        <is>
+          <t>11:40:00</t>
+        </is>
+      </c>
+      <c r="C201" s="4" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="D201" s="4" t="inlineStr"/>
+      <c r="E201" s="4" t="inlineStr"/>
+      <c r="F201" s="4" t="inlineStr"/>
+      <c r="G201" s="4" t="inlineStr"/>
+      <c r="H201" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I201" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J201" s="4" t="inlineStr"/>
+      <c r="K201" s="4" t="inlineStr"/>
+      <c r="L201" s="4" t="inlineStr"/>
+      <c r="M201" s="4" t="inlineStr"/>
+      <c r="N201" s="4" t="inlineStr"/>
+      <c r="O201" s="4" t="inlineStr"/>
+      <c r="P201" s="4" t="inlineStr">
         <is>
           <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
         </is>

</xml_diff>

<commit_message>
Update Oracle Cloud deployment script
- oracle_cloud_deploy_fixed.sh: Code formatting improvements and refinements
- Verified script syntax and deployment steps
- Ready for production deployment on Oracle Cloud Always Free Tier
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P201"/>
+  <dimension ref="A1:P203"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10224,6 +10224,90 @@
       <c r="N201" s="4" t="inlineStr"/>
       <c r="O201" s="4" t="inlineStr"/>
       <c r="P201" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:45:00</t>
+        </is>
+      </c>
+      <c r="B202" s="4" t="inlineStr">
+        <is>
+          <t>11:45:00</t>
+        </is>
+      </c>
+      <c r="C202" s="4" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D202" s="4" t="inlineStr"/>
+      <c r="E202" s="4" t="inlineStr"/>
+      <c r="F202" s="4" t="inlineStr"/>
+      <c r="G202" s="4" t="inlineStr"/>
+      <c r="H202" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I202" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J202" s="4" t="inlineStr"/>
+      <c r="K202" s="4" t="inlineStr"/>
+      <c r="L202" s="4" t="inlineStr"/>
+      <c r="M202" s="4" t="inlineStr"/>
+      <c r="N202" s="4" t="inlineStr"/>
+      <c r="O202" s="4" t="inlineStr"/>
+      <c r="P202" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:45:00</t>
+        </is>
+      </c>
+      <c r="B203" s="4" t="inlineStr">
+        <is>
+          <t>11:45:00</t>
+        </is>
+      </c>
+      <c r="C203" s="4" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D203" s="4" t="inlineStr"/>
+      <c r="E203" s="4" t="inlineStr"/>
+      <c r="F203" s="4" t="inlineStr"/>
+      <c r="G203" s="4" t="inlineStr"/>
+      <c r="H203" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I203" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J203" s="4" t="inlineStr"/>
+      <c r="K203" s="4" t="inlineStr"/>
+      <c r="L203" s="4" t="inlineStr"/>
+      <c r="M203" s="4" t="inlineStr"/>
+      <c r="N203" s="4" t="inlineStr"/>
+      <c r="O203" s="4" t="inlineStr"/>
+      <c r="P203" s="4" t="inlineStr">
         <is>
           <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
         </is>

</xml_diff>

<commit_message>
Add pytz dependency to pyproject.toml
</commit_message>
<xml_diff>
--- a/Mine/logs/mine_signal_logs.xlsx
+++ b/Mine/logs/mine_signal_logs.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P203"/>
+  <dimension ref="A1:P269"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10308,6 +10308,2778 @@
       <c r="N203" s="4" t="inlineStr"/>
       <c r="O203" s="4" t="inlineStr"/>
       <c r="P203" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:50:00</t>
+        </is>
+      </c>
+      <c r="B204" s="4" t="inlineStr">
+        <is>
+          <t>11:50:00</t>
+        </is>
+      </c>
+      <c r="C204" s="4" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="D204" s="4" t="inlineStr"/>
+      <c r="E204" s="4" t="inlineStr"/>
+      <c r="F204" s="4" t="inlineStr"/>
+      <c r="G204" s="4" t="inlineStr"/>
+      <c r="H204" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I204" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J204" s="4" t="inlineStr"/>
+      <c r="K204" s="4" t="inlineStr"/>
+      <c r="L204" s="4" t="inlineStr"/>
+      <c r="M204" s="4" t="inlineStr"/>
+      <c r="N204" s="4" t="inlineStr"/>
+      <c r="O204" s="4" t="inlineStr"/>
+      <c r="P204" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:50:00</t>
+        </is>
+      </c>
+      <c r="B205" s="4" t="inlineStr">
+        <is>
+          <t>11:50:00</t>
+        </is>
+      </c>
+      <c r="C205" s="4" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="D205" s="4" t="inlineStr"/>
+      <c r="E205" s="4" t="inlineStr"/>
+      <c r="F205" s="4" t="inlineStr"/>
+      <c r="G205" s="4" t="inlineStr"/>
+      <c r="H205" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I205" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J205" s="4" t="inlineStr"/>
+      <c r="K205" s="4" t="inlineStr"/>
+      <c r="L205" s="4" t="inlineStr"/>
+      <c r="M205" s="4" t="inlineStr"/>
+      <c r="N205" s="4" t="inlineStr"/>
+      <c r="O205" s="4" t="inlineStr"/>
+      <c r="P205" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:55:00</t>
+        </is>
+      </c>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t>11:55:00</t>
+        </is>
+      </c>
+      <c r="C206" s="4" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="D206" s="4" t="inlineStr"/>
+      <c r="E206" s="4" t="inlineStr"/>
+      <c r="F206" s="4" t="inlineStr"/>
+      <c r="G206" s="4" t="inlineStr"/>
+      <c r="H206" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I206" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J206" s="4" t="inlineStr"/>
+      <c r="K206" s="4" t="inlineStr"/>
+      <c r="L206" s="4" t="inlineStr"/>
+      <c r="M206" s="4" t="inlineStr"/>
+      <c r="N206" s="4" t="inlineStr"/>
+      <c r="O206" s="4" t="inlineStr"/>
+      <c r="P206" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 11:55:00</t>
+        </is>
+      </c>
+      <c r="B207" s="4" t="inlineStr">
+        <is>
+          <t>11:55:00</t>
+        </is>
+      </c>
+      <c r="C207" s="4" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="D207" s="4" t="inlineStr"/>
+      <c r="E207" s="4" t="inlineStr"/>
+      <c r="F207" s="4" t="inlineStr"/>
+      <c r="G207" s="4" t="inlineStr"/>
+      <c r="H207" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I207" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J207" s="4" t="inlineStr"/>
+      <c r="K207" s="4" t="inlineStr"/>
+      <c r="L207" s="4" t="inlineStr"/>
+      <c r="M207" s="4" t="inlineStr"/>
+      <c r="N207" s="4" t="inlineStr"/>
+      <c r="O207" s="4" t="inlineStr"/>
+      <c r="P207" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t>12:00:00</t>
+        </is>
+      </c>
+      <c r="C208" s="4" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D208" s="4" t="inlineStr"/>
+      <c r="E208" s="4" t="inlineStr"/>
+      <c r="F208" s="4" t="inlineStr"/>
+      <c r="G208" s="4" t="inlineStr"/>
+      <c r="H208" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I208" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J208" s="4" t="inlineStr"/>
+      <c r="K208" s="4" t="inlineStr"/>
+      <c r="L208" s="4" t="inlineStr"/>
+      <c r="M208" s="4" t="inlineStr"/>
+      <c r="N208" s="4" t="inlineStr"/>
+      <c r="O208" s="4" t="inlineStr"/>
+      <c r="P208" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="B209" s="4" t="inlineStr">
+        <is>
+          <t>12:00:00</t>
+        </is>
+      </c>
+      <c r="C209" s="4" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D209" s="4" t="inlineStr"/>
+      <c r="E209" s="4" t="inlineStr"/>
+      <c r="F209" s="4" t="inlineStr"/>
+      <c r="G209" s="4" t="inlineStr"/>
+      <c r="H209" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I209" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J209" s="4" t="inlineStr"/>
+      <c r="K209" s="4" t="inlineStr"/>
+      <c r="L209" s="4" t="inlineStr"/>
+      <c r="M209" s="4" t="inlineStr"/>
+      <c r="N209" s="4" t="inlineStr"/>
+      <c r="O209" s="4" t="inlineStr"/>
+      <c r="P209" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:05:00</t>
+        </is>
+      </c>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t>12:05:00</t>
+        </is>
+      </c>
+      <c r="C210" s="4" t="inlineStr">
+        <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="D210" s="4" t="inlineStr"/>
+      <c r="E210" s="4" t="inlineStr"/>
+      <c r="F210" s="4" t="inlineStr"/>
+      <c r="G210" s="4" t="inlineStr"/>
+      <c r="H210" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I210" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J210" s="4" t="inlineStr"/>
+      <c r="K210" s="4" t="inlineStr"/>
+      <c r="L210" s="4" t="inlineStr"/>
+      <c r="M210" s="4" t="inlineStr"/>
+      <c r="N210" s="4" t="inlineStr"/>
+      <c r="O210" s="4" t="inlineStr"/>
+      <c r="P210" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:05:00</t>
+        </is>
+      </c>
+      <c r="B211" s="4" t="inlineStr">
+        <is>
+          <t>12:05:00</t>
+        </is>
+      </c>
+      <c r="C211" s="4" t="inlineStr">
+        <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr"/>
+      <c r="E211" s="4" t="inlineStr"/>
+      <c r="F211" s="4" t="inlineStr"/>
+      <c r="G211" s="4" t="inlineStr"/>
+      <c r="H211" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I211" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J211" s="4" t="inlineStr"/>
+      <c r="K211" s="4" t="inlineStr"/>
+      <c r="L211" s="4" t="inlineStr"/>
+      <c r="M211" s="4" t="inlineStr"/>
+      <c r="N211" s="4" t="inlineStr"/>
+      <c r="O211" s="4" t="inlineStr"/>
+      <c r="P211" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:10:00</t>
+        </is>
+      </c>
+      <c r="B212" s="4" t="inlineStr">
+        <is>
+          <t>12:10:00</t>
+        </is>
+      </c>
+      <c r="C212" s="4" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="D212" s="4" t="inlineStr"/>
+      <c r="E212" s="4" t="inlineStr"/>
+      <c r="F212" s="4" t="inlineStr"/>
+      <c r="G212" s="4" t="inlineStr"/>
+      <c r="H212" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I212" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J212" s="4" t="inlineStr"/>
+      <c r="K212" s="4" t="inlineStr"/>
+      <c r="L212" s="4" t="inlineStr"/>
+      <c r="M212" s="4" t="inlineStr"/>
+      <c r="N212" s="4" t="inlineStr"/>
+      <c r="O212" s="4" t="inlineStr"/>
+      <c r="P212" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:10:00</t>
+        </is>
+      </c>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t>12:10:00</t>
+        </is>
+      </c>
+      <c r="C213" s="4" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="D213" s="4" t="inlineStr"/>
+      <c r="E213" s="4" t="inlineStr"/>
+      <c r="F213" s="4" t="inlineStr"/>
+      <c r="G213" s="4" t="inlineStr"/>
+      <c r="H213" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I213" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J213" s="4" t="inlineStr"/>
+      <c r="K213" s="4" t="inlineStr"/>
+      <c r="L213" s="4" t="inlineStr"/>
+      <c r="M213" s="4" t="inlineStr"/>
+      <c r="N213" s="4" t="inlineStr"/>
+      <c r="O213" s="4" t="inlineStr"/>
+      <c r="P213" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:15:00</t>
+        </is>
+      </c>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t>12:15:00</t>
+        </is>
+      </c>
+      <c r="C214" s="4" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D214" s="4" t="inlineStr"/>
+      <c r="E214" s="4" t="inlineStr"/>
+      <c r="F214" s="4" t="inlineStr"/>
+      <c r="G214" s="4" t="inlineStr"/>
+      <c r="H214" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I214" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J214" s="4" t="inlineStr"/>
+      <c r="K214" s="4" t="inlineStr"/>
+      <c r="L214" s="4" t="inlineStr"/>
+      <c r="M214" s="4" t="inlineStr"/>
+      <c r="N214" s="4" t="inlineStr"/>
+      <c r="O214" s="4" t="inlineStr"/>
+      <c r="P214" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:15:00</t>
+        </is>
+      </c>
+      <c r="B215" s="4" t="inlineStr">
+        <is>
+          <t>12:15:00</t>
+        </is>
+      </c>
+      <c r="C215" s="4" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D215" s="4" t="inlineStr"/>
+      <c r="E215" s="4" t="inlineStr"/>
+      <c r="F215" s="4" t="inlineStr"/>
+      <c r="G215" s="4" t="inlineStr"/>
+      <c r="H215" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I215" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J215" s="4" t="inlineStr"/>
+      <c r="K215" s="4" t="inlineStr"/>
+      <c r="L215" s="4" t="inlineStr"/>
+      <c r="M215" s="4" t="inlineStr"/>
+      <c r="N215" s="4" t="inlineStr"/>
+      <c r="O215" s="4" t="inlineStr"/>
+      <c r="P215" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:20:00</t>
+        </is>
+      </c>
+      <c r="B216" s="4" t="inlineStr">
+        <is>
+          <t>12:20:00</t>
+        </is>
+      </c>
+      <c r="C216" s="4" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="D216" s="4" t="inlineStr"/>
+      <c r="E216" s="4" t="inlineStr"/>
+      <c r="F216" s="4" t="inlineStr"/>
+      <c r="G216" s="4" t="inlineStr"/>
+      <c r="H216" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I216" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J216" s="4" t="inlineStr"/>
+      <c r="K216" s="4" t="inlineStr"/>
+      <c r="L216" s="4" t="inlineStr"/>
+      <c r="M216" s="4" t="inlineStr"/>
+      <c r="N216" s="4" t="inlineStr"/>
+      <c r="O216" s="4" t="inlineStr"/>
+      <c r="P216" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:20:00</t>
+        </is>
+      </c>
+      <c r="B217" s="4" t="inlineStr">
+        <is>
+          <t>12:20:00</t>
+        </is>
+      </c>
+      <c r="C217" s="4" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="D217" s="4" t="inlineStr"/>
+      <c r="E217" s="4" t="inlineStr"/>
+      <c r="F217" s="4" t="inlineStr"/>
+      <c r="G217" s="4" t="inlineStr"/>
+      <c r="H217" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I217" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J217" s="4" t="inlineStr"/>
+      <c r="K217" s="4" t="inlineStr"/>
+      <c r="L217" s="4" t="inlineStr"/>
+      <c r="M217" s="4" t="inlineStr"/>
+      <c r="N217" s="4" t="inlineStr"/>
+      <c r="O217" s="4" t="inlineStr"/>
+      <c r="P217" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:25:00</t>
+        </is>
+      </c>
+      <c r="B218" s="4" t="inlineStr">
+        <is>
+          <t>12:25:00</t>
+        </is>
+      </c>
+      <c r="C218" s="4" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="D218" s="4" t="inlineStr"/>
+      <c r="E218" s="4" t="inlineStr"/>
+      <c r="F218" s="4" t="inlineStr"/>
+      <c r="G218" s="4" t="inlineStr"/>
+      <c r="H218" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I218" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J218" s="4" t="inlineStr"/>
+      <c r="K218" s="4" t="inlineStr"/>
+      <c r="L218" s="4" t="inlineStr"/>
+      <c r="M218" s="4" t="inlineStr"/>
+      <c r="N218" s="4" t="inlineStr"/>
+      <c r="O218" s="4" t="inlineStr"/>
+      <c r="P218" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:25:00</t>
+        </is>
+      </c>
+      <c r="B219" s="4" t="inlineStr">
+        <is>
+          <t>12:25:00</t>
+        </is>
+      </c>
+      <c r="C219" s="4" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="D219" s="4" t="inlineStr"/>
+      <c r="E219" s="4" t="inlineStr"/>
+      <c r="F219" s="4" t="inlineStr"/>
+      <c r="G219" s="4" t="inlineStr"/>
+      <c r="H219" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I219" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J219" s="4" t="inlineStr"/>
+      <c r="K219" s="4" t="inlineStr"/>
+      <c r="L219" s="4" t="inlineStr"/>
+      <c r="M219" s="4" t="inlineStr"/>
+      <c r="N219" s="4" t="inlineStr"/>
+      <c r="O219" s="4" t="inlineStr"/>
+      <c r="P219" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:30:00</t>
+        </is>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="C220" s="4" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D220" s="4" t="inlineStr"/>
+      <c r="E220" s="4" t="inlineStr"/>
+      <c r="F220" s="4" t="inlineStr"/>
+      <c r="G220" s="4" t="inlineStr"/>
+      <c r="H220" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I220" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J220" s="4" t="inlineStr"/>
+      <c r="K220" s="4" t="inlineStr"/>
+      <c r="L220" s="4" t="inlineStr"/>
+      <c r="M220" s="4" t="inlineStr"/>
+      <c r="N220" s="4" t="inlineStr"/>
+      <c r="O220" s="4" t="inlineStr"/>
+      <c r="P220" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:30:00</t>
+        </is>
+      </c>
+      <c r="B221" s="4" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="C221" s="4" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D221" s="4" t="inlineStr"/>
+      <c r="E221" s="4" t="inlineStr"/>
+      <c r="F221" s="4" t="inlineStr"/>
+      <c r="G221" s="4" t="inlineStr"/>
+      <c r="H221" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I221" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J221" s="4" t="inlineStr"/>
+      <c r="K221" s="4" t="inlineStr"/>
+      <c r="L221" s="4" t="inlineStr"/>
+      <c r="M221" s="4" t="inlineStr"/>
+      <c r="N221" s="4" t="inlineStr"/>
+      <c r="O221" s="4" t="inlineStr"/>
+      <c r="P221" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:35:00</t>
+        </is>
+      </c>
+      <c r="B222" s="4" t="inlineStr">
+        <is>
+          <t>12:35:00</t>
+        </is>
+      </c>
+      <c r="C222" s="4" t="inlineStr">
+        <is>
+          <t>12:35</t>
+        </is>
+      </c>
+      <c r="D222" s="4" t="inlineStr"/>
+      <c r="E222" s="4" t="inlineStr"/>
+      <c r="F222" s="4" t="inlineStr"/>
+      <c r="G222" s="4" t="inlineStr"/>
+      <c r="H222" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I222" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J222" s="4" t="inlineStr"/>
+      <c r="K222" s="4" t="inlineStr"/>
+      <c r="L222" s="4" t="inlineStr"/>
+      <c r="M222" s="4" t="inlineStr"/>
+      <c r="N222" s="4" t="inlineStr"/>
+      <c r="O222" s="4" t="inlineStr"/>
+      <c r="P222" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:35:00</t>
+        </is>
+      </c>
+      <c r="B223" s="4" t="inlineStr">
+        <is>
+          <t>12:35:00</t>
+        </is>
+      </c>
+      <c r="C223" s="4" t="inlineStr">
+        <is>
+          <t>12:35</t>
+        </is>
+      </c>
+      <c r="D223" s="4" t="inlineStr"/>
+      <c r="E223" s="4" t="inlineStr"/>
+      <c r="F223" s="4" t="inlineStr"/>
+      <c r="G223" s="4" t="inlineStr"/>
+      <c r="H223" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I223" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J223" s="4" t="inlineStr"/>
+      <c r="K223" s="4" t="inlineStr"/>
+      <c r="L223" s="4" t="inlineStr"/>
+      <c r="M223" s="4" t="inlineStr"/>
+      <c r="N223" s="4" t="inlineStr"/>
+      <c r="O223" s="4" t="inlineStr"/>
+      <c r="P223" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:40:00</t>
+        </is>
+      </c>
+      <c r="B224" s="4" t="inlineStr">
+        <is>
+          <t>12:40:00</t>
+        </is>
+      </c>
+      <c r="C224" s="4" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="D224" s="4" t="inlineStr"/>
+      <c r="E224" s="4" t="inlineStr"/>
+      <c r="F224" s="4" t="inlineStr"/>
+      <c r="G224" s="4" t="inlineStr"/>
+      <c r="H224" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I224" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J224" s="4" t="inlineStr"/>
+      <c r="K224" s="4" t="inlineStr"/>
+      <c r="L224" s="4" t="inlineStr"/>
+      <c r="M224" s="4" t="inlineStr"/>
+      <c r="N224" s="4" t="inlineStr"/>
+      <c r="O224" s="4" t="inlineStr"/>
+      <c r="P224" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:40:00</t>
+        </is>
+      </c>
+      <c r="B225" s="4" t="inlineStr">
+        <is>
+          <t>12:40:00</t>
+        </is>
+      </c>
+      <c r="C225" s="4" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="D225" s="4" t="inlineStr"/>
+      <c r="E225" s="4" t="inlineStr"/>
+      <c r="F225" s="4" t="inlineStr"/>
+      <c r="G225" s="4" t="inlineStr"/>
+      <c r="H225" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I225" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J225" s="4" t="inlineStr"/>
+      <c r="K225" s="4" t="inlineStr"/>
+      <c r="L225" s="4" t="inlineStr"/>
+      <c r="M225" s="4" t="inlineStr"/>
+      <c r="N225" s="4" t="inlineStr"/>
+      <c r="O225" s="4" t="inlineStr"/>
+      <c r="P225" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:45:00</t>
+        </is>
+      </c>
+      <c r="B226" s="4" t="inlineStr">
+        <is>
+          <t>12:45:00</t>
+        </is>
+      </c>
+      <c r="C226" s="4" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D226" s="4" t="inlineStr"/>
+      <c r="E226" s="4" t="inlineStr"/>
+      <c r="F226" s="4" t="inlineStr"/>
+      <c r="G226" s="4" t="inlineStr"/>
+      <c r="H226" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I226" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J226" s="4" t="inlineStr"/>
+      <c r="K226" s="4" t="inlineStr"/>
+      <c r="L226" s="4" t="inlineStr"/>
+      <c r="M226" s="4" t="inlineStr"/>
+      <c r="N226" s="4" t="inlineStr"/>
+      <c r="O226" s="4" t="inlineStr"/>
+      <c r="P226" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:45:00</t>
+        </is>
+      </c>
+      <c r="B227" s="4" t="inlineStr">
+        <is>
+          <t>12:45:00</t>
+        </is>
+      </c>
+      <c r="C227" s="4" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D227" s="4" t="inlineStr"/>
+      <c r="E227" s="4" t="inlineStr"/>
+      <c r="F227" s="4" t="inlineStr"/>
+      <c r="G227" s="4" t="inlineStr"/>
+      <c r="H227" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I227" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J227" s="4" t="inlineStr"/>
+      <c r="K227" s="4" t="inlineStr"/>
+      <c r="L227" s="4" t="inlineStr"/>
+      <c r="M227" s="4" t="inlineStr"/>
+      <c r="N227" s="4" t="inlineStr"/>
+      <c r="O227" s="4" t="inlineStr"/>
+      <c r="P227" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:50:00</t>
+        </is>
+      </c>
+      <c r="B228" s="4" t="inlineStr">
+        <is>
+          <t>12:50:00</t>
+        </is>
+      </c>
+      <c r="C228" s="4" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="D228" s="4" t="inlineStr"/>
+      <c r="E228" s="4" t="inlineStr"/>
+      <c r="F228" s="4" t="inlineStr"/>
+      <c r="G228" s="4" t="inlineStr"/>
+      <c r="H228" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I228" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J228" s="4" t="inlineStr"/>
+      <c r="K228" s="4" t="inlineStr"/>
+      <c r="L228" s="4" t="inlineStr"/>
+      <c r="M228" s="4" t="inlineStr"/>
+      <c r="N228" s="4" t="inlineStr"/>
+      <c r="O228" s="4" t="inlineStr"/>
+      <c r="P228" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:50:00</t>
+        </is>
+      </c>
+      <c r="B229" s="4" t="inlineStr">
+        <is>
+          <t>12:50:00</t>
+        </is>
+      </c>
+      <c r="C229" s="4" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="D229" s="4" t="inlineStr"/>
+      <c r="E229" s="4" t="inlineStr"/>
+      <c r="F229" s="4" t="inlineStr"/>
+      <c r="G229" s="4" t="inlineStr"/>
+      <c r="H229" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I229" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J229" s="4" t="inlineStr"/>
+      <c r="K229" s="4" t="inlineStr"/>
+      <c r="L229" s="4" t="inlineStr"/>
+      <c r="M229" s="4" t="inlineStr"/>
+      <c r="N229" s="4" t="inlineStr"/>
+      <c r="O229" s="4" t="inlineStr"/>
+      <c r="P229" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:55:00</t>
+        </is>
+      </c>
+      <c r="B230" s="4" t="inlineStr">
+        <is>
+          <t>12:55:00</t>
+        </is>
+      </c>
+      <c r="C230" s="4" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="D230" s="4" t="inlineStr"/>
+      <c r="E230" s="4" t="inlineStr"/>
+      <c r="F230" s="4" t="inlineStr"/>
+      <c r="G230" s="4" t="inlineStr"/>
+      <c r="H230" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I230" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J230" s="4" t="inlineStr"/>
+      <c r="K230" s="4" t="inlineStr"/>
+      <c r="L230" s="4" t="inlineStr"/>
+      <c r="M230" s="4" t="inlineStr"/>
+      <c r="N230" s="4" t="inlineStr"/>
+      <c r="O230" s="4" t="inlineStr"/>
+      <c r="P230" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 12:55:00</t>
+        </is>
+      </c>
+      <c r="B231" s="4" t="inlineStr">
+        <is>
+          <t>12:55:00</t>
+        </is>
+      </c>
+      <c r="C231" s="4" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="D231" s="4" t="inlineStr"/>
+      <c r="E231" s="4" t="inlineStr"/>
+      <c r="F231" s="4" t="inlineStr"/>
+      <c r="G231" s="4" t="inlineStr"/>
+      <c r="H231" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I231" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J231" s="4" t="inlineStr"/>
+      <c r="K231" s="4" t="inlineStr"/>
+      <c r="L231" s="4" t="inlineStr"/>
+      <c r="M231" s="4" t="inlineStr"/>
+      <c r="N231" s="4" t="inlineStr"/>
+      <c r="O231" s="4" t="inlineStr"/>
+      <c r="P231" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:00:00</t>
+        </is>
+      </c>
+      <c r="B232" s="4" t="inlineStr">
+        <is>
+          <t>13:00:00</t>
+        </is>
+      </c>
+      <c r="C232" s="4" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D232" s="4" t="inlineStr"/>
+      <c r="E232" s="4" t="inlineStr"/>
+      <c r="F232" s="4" t="inlineStr"/>
+      <c r="G232" s="4" t="inlineStr"/>
+      <c r="H232" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I232" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J232" s="4" t="inlineStr"/>
+      <c r="K232" s="4" t="inlineStr"/>
+      <c r="L232" s="4" t="inlineStr"/>
+      <c r="M232" s="4" t="inlineStr"/>
+      <c r="N232" s="4" t="inlineStr"/>
+      <c r="O232" s="4" t="inlineStr"/>
+      <c r="P232" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:00:00</t>
+        </is>
+      </c>
+      <c r="B233" s="4" t="inlineStr">
+        <is>
+          <t>13:00:00</t>
+        </is>
+      </c>
+      <c r="C233" s="4" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D233" s="4" t="inlineStr"/>
+      <c r="E233" s="4" t="inlineStr"/>
+      <c r="F233" s="4" t="inlineStr"/>
+      <c r="G233" s="4" t="inlineStr"/>
+      <c r="H233" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I233" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J233" s="4" t="inlineStr"/>
+      <c r="K233" s="4" t="inlineStr"/>
+      <c r="L233" s="4" t="inlineStr"/>
+      <c r="M233" s="4" t="inlineStr"/>
+      <c r="N233" s="4" t="inlineStr"/>
+      <c r="O233" s="4" t="inlineStr"/>
+      <c r="P233" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:35:00</t>
+        </is>
+      </c>
+      <c r="B234" s="4" t="inlineStr">
+        <is>
+          <t>13:35:00</t>
+        </is>
+      </c>
+      <c r="C234" s="4" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="D234" s="4" t="inlineStr"/>
+      <c r="E234" s="4" t="inlineStr"/>
+      <c r="F234" s="4" t="inlineStr"/>
+      <c r="G234" s="4" t="inlineStr"/>
+      <c r="H234" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I234" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J234" s="4" t="inlineStr"/>
+      <c r="K234" s="4" t="inlineStr"/>
+      <c r="L234" s="4" t="inlineStr"/>
+      <c r="M234" s="4" t="inlineStr"/>
+      <c r="N234" s="4" t="inlineStr"/>
+      <c r="O234" s="4" t="inlineStr"/>
+      <c r="P234" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:35:00</t>
+        </is>
+      </c>
+      <c r="B235" s="4" t="inlineStr">
+        <is>
+          <t>13:35:00</t>
+        </is>
+      </c>
+      <c r="C235" s="4" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="D235" s="4" t="inlineStr"/>
+      <c r="E235" s="4" t="inlineStr"/>
+      <c r="F235" s="4" t="inlineStr"/>
+      <c r="G235" s="4" t="inlineStr"/>
+      <c r="H235" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I235" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J235" s="4" t="inlineStr"/>
+      <c r="K235" s="4" t="inlineStr"/>
+      <c r="L235" s="4" t="inlineStr"/>
+      <c r="M235" s="4" t="inlineStr"/>
+      <c r="N235" s="4" t="inlineStr"/>
+      <c r="O235" s="4" t="inlineStr"/>
+      <c r="P235" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:40:00</t>
+        </is>
+      </c>
+      <c r="B236" s="4" t="inlineStr">
+        <is>
+          <t>13:40:00</t>
+        </is>
+      </c>
+      <c r="C236" s="4" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="D236" s="4" t="inlineStr"/>
+      <c r="E236" s="4" t="inlineStr"/>
+      <c r="F236" s="4" t="inlineStr"/>
+      <c r="G236" s="4" t="inlineStr"/>
+      <c r="H236" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I236" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J236" s="4" t="inlineStr"/>
+      <c r="K236" s="4" t="inlineStr"/>
+      <c r="L236" s="4" t="inlineStr"/>
+      <c r="M236" s="4" t="inlineStr"/>
+      <c r="N236" s="4" t="inlineStr"/>
+      <c r="O236" s="4" t="inlineStr"/>
+      <c r="P236" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:40:00</t>
+        </is>
+      </c>
+      <c r="B237" s="4" t="inlineStr">
+        <is>
+          <t>13:40:00</t>
+        </is>
+      </c>
+      <c r="C237" s="4" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="D237" s="4" t="inlineStr"/>
+      <c r="E237" s="4" t="inlineStr"/>
+      <c r="F237" s="4" t="inlineStr"/>
+      <c r="G237" s="4" t="inlineStr"/>
+      <c r="H237" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I237" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J237" s="4" t="inlineStr"/>
+      <c r="K237" s="4" t="inlineStr"/>
+      <c r="L237" s="4" t="inlineStr"/>
+      <c r="M237" s="4" t="inlineStr"/>
+      <c r="N237" s="4" t="inlineStr"/>
+      <c r="O237" s="4" t="inlineStr"/>
+      <c r="P237" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:45:00</t>
+        </is>
+      </c>
+      <c r="B238" s="4" t="inlineStr">
+        <is>
+          <t>13:45:00</t>
+        </is>
+      </c>
+      <c r="C238" s="4" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D238" s="4" t="inlineStr"/>
+      <c r="E238" s="4" t="inlineStr"/>
+      <c r="F238" s="4" t="inlineStr"/>
+      <c r="G238" s="4" t="inlineStr"/>
+      <c r="H238" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I238" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J238" s="4" t="inlineStr"/>
+      <c r="K238" s="4" t="inlineStr"/>
+      <c r="L238" s="4" t="inlineStr"/>
+      <c r="M238" s="4" t="inlineStr"/>
+      <c r="N238" s="4" t="inlineStr"/>
+      <c r="O238" s="4" t="inlineStr"/>
+      <c r="P238" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:45:00</t>
+        </is>
+      </c>
+      <c r="B239" s="4" t="inlineStr">
+        <is>
+          <t>13:45:00</t>
+        </is>
+      </c>
+      <c r="C239" s="4" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D239" s="4" t="inlineStr"/>
+      <c r="E239" s="4" t="inlineStr"/>
+      <c r="F239" s="4" t="inlineStr"/>
+      <c r="G239" s="4" t="inlineStr"/>
+      <c r="H239" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I239" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J239" s="4" t="inlineStr"/>
+      <c r="K239" s="4" t="inlineStr"/>
+      <c r="L239" s="4" t="inlineStr"/>
+      <c r="M239" s="4" t="inlineStr"/>
+      <c r="N239" s="4" t="inlineStr"/>
+      <c r="O239" s="4" t="inlineStr"/>
+      <c r="P239" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:50:00</t>
+        </is>
+      </c>
+      <c r="B240" s="4" t="inlineStr">
+        <is>
+          <t>13:50:00</t>
+        </is>
+      </c>
+      <c r="C240" s="4" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="D240" s="4" t="inlineStr"/>
+      <c r="E240" s="4" t="inlineStr"/>
+      <c r="F240" s="4" t="inlineStr"/>
+      <c r="G240" s="4" t="inlineStr"/>
+      <c r="H240" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I240" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J240" s="4" t="inlineStr"/>
+      <c r="K240" s="4" t="inlineStr"/>
+      <c r="L240" s="4" t="inlineStr"/>
+      <c r="M240" s="4" t="inlineStr"/>
+      <c r="N240" s="4" t="inlineStr"/>
+      <c r="O240" s="4" t="inlineStr"/>
+      <c r="P240" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:50:00</t>
+        </is>
+      </c>
+      <c r="B241" s="4" t="inlineStr">
+        <is>
+          <t>13:50:00</t>
+        </is>
+      </c>
+      <c r="C241" s="4" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="D241" s="4" t="inlineStr"/>
+      <c r="E241" s="4" t="inlineStr"/>
+      <c r="F241" s="4" t="inlineStr"/>
+      <c r="G241" s="4" t="inlineStr"/>
+      <c r="H241" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I241" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J241" s="4" t="inlineStr"/>
+      <c r="K241" s="4" t="inlineStr"/>
+      <c r="L241" s="4" t="inlineStr"/>
+      <c r="M241" s="4" t="inlineStr"/>
+      <c r="N241" s="4" t="inlineStr"/>
+      <c r="O241" s="4" t="inlineStr"/>
+      <c r="P241" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:55:00</t>
+        </is>
+      </c>
+      <c r="B242" s="4" t="inlineStr">
+        <is>
+          <t>13:55:00</t>
+        </is>
+      </c>
+      <c r="C242" s="4" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="D242" s="4" t="inlineStr"/>
+      <c r="E242" s="4" t="inlineStr"/>
+      <c r="F242" s="4" t="inlineStr"/>
+      <c r="G242" s="4" t="inlineStr"/>
+      <c r="H242" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I242" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J242" s="4" t="inlineStr"/>
+      <c r="K242" s="4" t="inlineStr"/>
+      <c r="L242" s="4" t="inlineStr"/>
+      <c r="M242" s="4" t="inlineStr"/>
+      <c r="N242" s="4" t="inlineStr"/>
+      <c r="O242" s="4" t="inlineStr"/>
+      <c r="P242" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 13:55:00</t>
+        </is>
+      </c>
+      <c r="B243" s="4" t="inlineStr">
+        <is>
+          <t>13:55:00</t>
+        </is>
+      </c>
+      <c r="C243" s="4" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="D243" s="4" t="inlineStr"/>
+      <c r="E243" s="4" t="inlineStr"/>
+      <c r="F243" s="4" t="inlineStr"/>
+      <c r="G243" s="4" t="inlineStr"/>
+      <c r="H243" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I243" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J243" s="4" t="inlineStr"/>
+      <c r="K243" s="4" t="inlineStr"/>
+      <c r="L243" s="4" t="inlineStr"/>
+      <c r="M243" s="4" t="inlineStr"/>
+      <c r="N243" s="4" t="inlineStr"/>
+      <c r="O243" s="4" t="inlineStr"/>
+      <c r="P243" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="B244" s="4" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="C244" s="4" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D244" s="4" t="inlineStr"/>
+      <c r="E244" s="4" t="inlineStr"/>
+      <c r="F244" s="4" t="inlineStr"/>
+      <c r="G244" s="4" t="inlineStr"/>
+      <c r="H244" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I244" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J244" s="4" t="inlineStr"/>
+      <c r="K244" s="4" t="inlineStr"/>
+      <c r="L244" s="4" t="inlineStr"/>
+      <c r="M244" s="4" t="inlineStr"/>
+      <c r="N244" s="4" t="inlineStr"/>
+      <c r="O244" s="4" t="inlineStr"/>
+      <c r="P244" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="B245" s="4" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="C245" s="4" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D245" s="4" t="inlineStr"/>
+      <c r="E245" s="4" t="inlineStr"/>
+      <c r="F245" s="4" t="inlineStr"/>
+      <c r="G245" s="4" t="inlineStr"/>
+      <c r="H245" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I245" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J245" s="4" t="inlineStr"/>
+      <c r="K245" s="4" t="inlineStr"/>
+      <c r="L245" s="4" t="inlineStr"/>
+      <c r="M245" s="4" t="inlineStr"/>
+      <c r="N245" s="4" t="inlineStr"/>
+      <c r="O245" s="4" t="inlineStr"/>
+      <c r="P245" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05:00</t>
+        </is>
+      </c>
+      <c r="B246" s="4" t="inlineStr">
+        <is>
+          <t>14:05:00</t>
+        </is>
+      </c>
+      <c r="C246" s="4" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="D246" s="4" t="inlineStr"/>
+      <c r="E246" s="4" t="inlineStr"/>
+      <c r="F246" s="4" t="inlineStr"/>
+      <c r="G246" s="4" t="inlineStr"/>
+      <c r="H246" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I246" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J246" s="4" t="inlineStr"/>
+      <c r="K246" s="4" t="inlineStr"/>
+      <c r="L246" s="4" t="inlineStr"/>
+      <c r="M246" s="4" t="inlineStr"/>
+      <c r="N246" s="4" t="inlineStr"/>
+      <c r="O246" s="4" t="inlineStr"/>
+      <c r="P246" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:05:00</t>
+        </is>
+      </c>
+      <c r="B247" s="4" t="inlineStr">
+        <is>
+          <t>14:05:00</t>
+        </is>
+      </c>
+      <c r="C247" s="4" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="D247" s="4" t="inlineStr"/>
+      <c r="E247" s="4" t="inlineStr"/>
+      <c r="F247" s="4" t="inlineStr"/>
+      <c r="G247" s="4" t="inlineStr"/>
+      <c r="H247" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I247" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J247" s="4" t="inlineStr"/>
+      <c r="K247" s="4" t="inlineStr"/>
+      <c r="L247" s="4" t="inlineStr"/>
+      <c r="M247" s="4" t="inlineStr"/>
+      <c r="N247" s="4" t="inlineStr"/>
+      <c r="O247" s="4" t="inlineStr"/>
+      <c r="P247" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:10:00</t>
+        </is>
+      </c>
+      <c r="B248" s="4" t="inlineStr">
+        <is>
+          <t>14:10:00</t>
+        </is>
+      </c>
+      <c r="C248" s="4" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="D248" s="4" t="inlineStr"/>
+      <c r="E248" s="4" t="inlineStr"/>
+      <c r="F248" s="4" t="inlineStr"/>
+      <c r="G248" s="4" t="inlineStr"/>
+      <c r="H248" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I248" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J248" s="4" t="inlineStr"/>
+      <c r="K248" s="4" t="inlineStr"/>
+      <c r="L248" s="4" t="inlineStr"/>
+      <c r="M248" s="4" t="inlineStr"/>
+      <c r="N248" s="4" t="inlineStr"/>
+      <c r="O248" s="4" t="inlineStr"/>
+      <c r="P248" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:10:00</t>
+        </is>
+      </c>
+      <c r="B249" s="4" t="inlineStr">
+        <is>
+          <t>14:10:00</t>
+        </is>
+      </c>
+      <c r="C249" s="4" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="D249" s="4" t="inlineStr"/>
+      <c r="E249" s="4" t="inlineStr"/>
+      <c r="F249" s="4" t="inlineStr"/>
+      <c r="G249" s="4" t="inlineStr"/>
+      <c r="H249" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I249" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J249" s="4" t="inlineStr"/>
+      <c r="K249" s="4" t="inlineStr"/>
+      <c r="L249" s="4" t="inlineStr"/>
+      <c r="M249" s="4" t="inlineStr"/>
+      <c r="N249" s="4" t="inlineStr"/>
+      <c r="O249" s="4" t="inlineStr"/>
+      <c r="P249" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:15:00</t>
+        </is>
+      </c>
+      <c r="B250" s="4" t="inlineStr">
+        <is>
+          <t>14:15:00</t>
+        </is>
+      </c>
+      <c r="C250" s="4" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="D250" s="4" t="inlineStr"/>
+      <c r="E250" s="4" t="inlineStr"/>
+      <c r="F250" s="4" t="inlineStr"/>
+      <c r="G250" s="4" t="inlineStr"/>
+      <c r="H250" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I250" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J250" s="4" t="inlineStr"/>
+      <c r="K250" s="4" t="inlineStr"/>
+      <c r="L250" s="4" t="inlineStr"/>
+      <c r="M250" s="4" t="inlineStr"/>
+      <c r="N250" s="4" t="inlineStr"/>
+      <c r="O250" s="4" t="inlineStr"/>
+      <c r="P250" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:15:00</t>
+        </is>
+      </c>
+      <c r="B251" s="4" t="inlineStr">
+        <is>
+          <t>14:15:00</t>
+        </is>
+      </c>
+      <c r="C251" s="4" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="D251" s="4" t="inlineStr"/>
+      <c r="E251" s="4" t="inlineStr"/>
+      <c r="F251" s="4" t="inlineStr"/>
+      <c r="G251" s="4" t="inlineStr"/>
+      <c r="H251" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I251" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J251" s="4" t="inlineStr"/>
+      <c r="K251" s="4" t="inlineStr"/>
+      <c r="L251" s="4" t="inlineStr"/>
+      <c r="M251" s="4" t="inlineStr"/>
+      <c r="N251" s="4" t="inlineStr"/>
+      <c r="O251" s="4" t="inlineStr"/>
+      <c r="P251" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:20:00</t>
+        </is>
+      </c>
+      <c r="B252" s="4" t="inlineStr">
+        <is>
+          <t>14:20:00</t>
+        </is>
+      </c>
+      <c r="C252" s="4" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="D252" s="4" t="inlineStr"/>
+      <c r="E252" s="4" t="inlineStr"/>
+      <c r="F252" s="4" t="inlineStr"/>
+      <c r="G252" s="4" t="inlineStr"/>
+      <c r="H252" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I252" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J252" s="4" t="inlineStr"/>
+      <c r="K252" s="4" t="inlineStr"/>
+      <c r="L252" s="4" t="inlineStr"/>
+      <c r="M252" s="4" t="inlineStr"/>
+      <c r="N252" s="4" t="inlineStr"/>
+      <c r="O252" s="4" t="inlineStr"/>
+      <c r="P252" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:20:00</t>
+        </is>
+      </c>
+      <c r="B253" s="4" t="inlineStr">
+        <is>
+          <t>14:20:00</t>
+        </is>
+      </c>
+      <c r="C253" s="4" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="D253" s="4" t="inlineStr"/>
+      <c r="E253" s="4" t="inlineStr"/>
+      <c r="F253" s="4" t="inlineStr"/>
+      <c r="G253" s="4" t="inlineStr"/>
+      <c r="H253" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I253" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J253" s="4" t="inlineStr"/>
+      <c r="K253" s="4" t="inlineStr"/>
+      <c r="L253" s="4" t="inlineStr"/>
+      <c r="M253" s="4" t="inlineStr"/>
+      <c r="N253" s="4" t="inlineStr"/>
+      <c r="O253" s="4" t="inlineStr"/>
+      <c r="P253" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:25:00</t>
+        </is>
+      </c>
+      <c r="B254" s="4" t="inlineStr">
+        <is>
+          <t>14:25:00</t>
+        </is>
+      </c>
+      <c r="C254" s="4" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="D254" s="4" t="inlineStr"/>
+      <c r="E254" s="4" t="inlineStr"/>
+      <c r="F254" s="4" t="inlineStr"/>
+      <c r="G254" s="4" t="inlineStr"/>
+      <c r="H254" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I254" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J254" s="4" t="inlineStr"/>
+      <c r="K254" s="4" t="inlineStr"/>
+      <c r="L254" s="4" t="inlineStr"/>
+      <c r="M254" s="4" t="inlineStr"/>
+      <c r="N254" s="4" t="inlineStr"/>
+      <c r="O254" s="4" t="inlineStr"/>
+      <c r="P254" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:25:00</t>
+        </is>
+      </c>
+      <c r="B255" s="4" t="inlineStr">
+        <is>
+          <t>14:25:00</t>
+        </is>
+      </c>
+      <c r="C255" s="4" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="D255" s="4" t="inlineStr"/>
+      <c r="E255" s="4" t="inlineStr"/>
+      <c r="F255" s="4" t="inlineStr"/>
+      <c r="G255" s="4" t="inlineStr"/>
+      <c r="H255" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I255" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J255" s="4" t="inlineStr"/>
+      <c r="K255" s="4" t="inlineStr"/>
+      <c r="L255" s="4" t="inlineStr"/>
+      <c r="M255" s="4" t="inlineStr"/>
+      <c r="N255" s="4" t="inlineStr"/>
+      <c r="O255" s="4" t="inlineStr"/>
+      <c r="P255" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:30:00</t>
+        </is>
+      </c>
+      <c r="B256" s="4" t="inlineStr">
+        <is>
+          <t>14:30:00</t>
+        </is>
+      </c>
+      <c r="C256" s="4" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D256" s="4" t="inlineStr"/>
+      <c r="E256" s="4" t="inlineStr"/>
+      <c r="F256" s="4" t="inlineStr"/>
+      <c r="G256" s="4" t="inlineStr"/>
+      <c r="H256" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I256" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J256" s="4" t="inlineStr"/>
+      <c r="K256" s="4" t="inlineStr"/>
+      <c r="L256" s="4" t="inlineStr"/>
+      <c r="M256" s="4" t="inlineStr"/>
+      <c r="N256" s="4" t="inlineStr"/>
+      <c r="O256" s="4" t="inlineStr"/>
+      <c r="P256" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:30:00</t>
+        </is>
+      </c>
+      <c r="B257" s="4" t="inlineStr">
+        <is>
+          <t>14:30:00</t>
+        </is>
+      </c>
+      <c r="C257" s="4" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D257" s="4" t="inlineStr"/>
+      <c r="E257" s="4" t="inlineStr"/>
+      <c r="F257" s="4" t="inlineStr"/>
+      <c r="G257" s="4" t="inlineStr"/>
+      <c r="H257" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I257" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J257" s="4" t="inlineStr"/>
+      <c r="K257" s="4" t="inlineStr"/>
+      <c r="L257" s="4" t="inlineStr"/>
+      <c r="M257" s="4" t="inlineStr"/>
+      <c r="N257" s="4" t="inlineStr"/>
+      <c r="O257" s="4" t="inlineStr"/>
+      <c r="P257" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:35:00</t>
+        </is>
+      </c>
+      <c r="B258" s="4" t="inlineStr">
+        <is>
+          <t>14:35:00</t>
+        </is>
+      </c>
+      <c r="C258" s="4" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="D258" s="4" t="inlineStr"/>
+      <c r="E258" s="4" t="inlineStr"/>
+      <c r="F258" s="4" t="inlineStr"/>
+      <c r="G258" s="4" t="inlineStr"/>
+      <c r="H258" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I258" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J258" s="4" t="inlineStr"/>
+      <c r="K258" s="4" t="inlineStr"/>
+      <c r="L258" s="4" t="inlineStr"/>
+      <c r="M258" s="4" t="inlineStr"/>
+      <c r="N258" s="4" t="inlineStr"/>
+      <c r="O258" s="4" t="inlineStr"/>
+      <c r="P258" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:35:00</t>
+        </is>
+      </c>
+      <c r="B259" s="4" t="inlineStr">
+        <is>
+          <t>14:35:00</t>
+        </is>
+      </c>
+      <c r="C259" s="4" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="D259" s="4" t="inlineStr"/>
+      <c r="E259" s="4" t="inlineStr"/>
+      <c r="F259" s="4" t="inlineStr"/>
+      <c r="G259" s="4" t="inlineStr"/>
+      <c r="H259" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I259" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J259" s="4" t="inlineStr"/>
+      <c r="K259" s="4" t="inlineStr"/>
+      <c r="L259" s="4" t="inlineStr"/>
+      <c r="M259" s="4" t="inlineStr"/>
+      <c r="N259" s="4" t="inlineStr"/>
+      <c r="O259" s="4" t="inlineStr"/>
+      <c r="P259" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:40:00</t>
+        </is>
+      </c>
+      <c r="B260" s="4" t="inlineStr">
+        <is>
+          <t>14:40:00</t>
+        </is>
+      </c>
+      <c r="C260" s="4" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="D260" s="4" t="inlineStr"/>
+      <c r="E260" s="4" t="inlineStr"/>
+      <c r="F260" s="4" t="inlineStr"/>
+      <c r="G260" s="4" t="inlineStr"/>
+      <c r="H260" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I260" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J260" s="4" t="inlineStr"/>
+      <c r="K260" s="4" t="inlineStr"/>
+      <c r="L260" s="4" t="inlineStr"/>
+      <c r="M260" s="4" t="inlineStr"/>
+      <c r="N260" s="4" t="inlineStr"/>
+      <c r="O260" s="4" t="inlineStr"/>
+      <c r="P260" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:40:00</t>
+        </is>
+      </c>
+      <c r="B261" s="4" t="inlineStr">
+        <is>
+          <t>14:40:00</t>
+        </is>
+      </c>
+      <c r="C261" s="4" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="D261" s="4" t="inlineStr"/>
+      <c r="E261" s="4" t="inlineStr"/>
+      <c r="F261" s="4" t="inlineStr"/>
+      <c r="G261" s="4" t="inlineStr"/>
+      <c r="H261" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I261" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J261" s="4" t="inlineStr"/>
+      <c r="K261" s="4" t="inlineStr"/>
+      <c r="L261" s="4" t="inlineStr"/>
+      <c r="M261" s="4" t="inlineStr"/>
+      <c r="N261" s="4" t="inlineStr"/>
+      <c r="O261" s="4" t="inlineStr"/>
+      <c r="P261" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:45:00</t>
+        </is>
+      </c>
+      <c r="B262" s="4" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="C262" s="4" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D262" s="4" t="inlineStr"/>
+      <c r="E262" s="4" t="inlineStr"/>
+      <c r="F262" s="4" t="inlineStr"/>
+      <c r="G262" s="4" t="inlineStr"/>
+      <c r="H262" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I262" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J262" s="4" t="inlineStr"/>
+      <c r="K262" s="4" t="inlineStr"/>
+      <c r="L262" s="4" t="inlineStr"/>
+      <c r="M262" s="4" t="inlineStr"/>
+      <c r="N262" s="4" t="inlineStr"/>
+      <c r="O262" s="4" t="inlineStr"/>
+      <c r="P262" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:45:00</t>
+        </is>
+      </c>
+      <c r="B263" s="4" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="C263" s="4" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D263" s="4" t="inlineStr"/>
+      <c r="E263" s="4" t="inlineStr"/>
+      <c r="F263" s="4" t="inlineStr"/>
+      <c r="G263" s="4" t="inlineStr"/>
+      <c r="H263" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I263" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J263" s="4" t="inlineStr"/>
+      <c r="K263" s="4" t="inlineStr"/>
+      <c r="L263" s="4" t="inlineStr"/>
+      <c r="M263" s="4" t="inlineStr"/>
+      <c r="N263" s="4" t="inlineStr"/>
+      <c r="O263" s="4" t="inlineStr"/>
+      <c r="P263" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:50:00</t>
+        </is>
+      </c>
+      <c r="B264" s="4" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C264" s="4" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D264" s="4" t="inlineStr"/>
+      <c r="E264" s="4" t="inlineStr"/>
+      <c r="F264" s="4" t="inlineStr"/>
+      <c r="G264" s="4" t="inlineStr"/>
+      <c r="H264" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I264" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J264" s="4" t="inlineStr"/>
+      <c r="K264" s="4" t="inlineStr"/>
+      <c r="L264" s="4" t="inlineStr"/>
+      <c r="M264" s="4" t="inlineStr"/>
+      <c r="N264" s="4" t="inlineStr"/>
+      <c r="O264" s="4" t="inlineStr"/>
+      <c r="P264" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:50:00</t>
+        </is>
+      </c>
+      <c r="B265" s="4" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C265" s="4" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D265" s="4" t="inlineStr"/>
+      <c r="E265" s="4" t="inlineStr"/>
+      <c r="F265" s="4" t="inlineStr"/>
+      <c r="G265" s="4" t="inlineStr"/>
+      <c r="H265" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I265" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J265" s="4" t="inlineStr"/>
+      <c r="K265" s="4" t="inlineStr"/>
+      <c r="L265" s="4" t="inlineStr"/>
+      <c r="M265" s="4" t="inlineStr"/>
+      <c r="N265" s="4" t="inlineStr"/>
+      <c r="O265" s="4" t="inlineStr"/>
+      <c r="P265" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:55:00</t>
+        </is>
+      </c>
+      <c r="B266" s="4" t="inlineStr">
+        <is>
+          <t>14:55:00</t>
+        </is>
+      </c>
+      <c r="C266" s="4" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="D266" s="4" t="inlineStr"/>
+      <c r="E266" s="4" t="inlineStr"/>
+      <c r="F266" s="4" t="inlineStr"/>
+      <c r="G266" s="4" t="inlineStr"/>
+      <c r="H266" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I266" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J266" s="4" t="inlineStr"/>
+      <c r="K266" s="4" t="inlineStr"/>
+      <c r="L266" s="4" t="inlineStr"/>
+      <c r="M266" s="4" t="inlineStr"/>
+      <c r="N266" s="4" t="inlineStr"/>
+      <c r="O266" s="4" t="inlineStr"/>
+      <c r="P266" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 14:55:00</t>
+        </is>
+      </c>
+      <c r="B267" s="4" t="inlineStr">
+        <is>
+          <t>14:55:00</t>
+        </is>
+      </c>
+      <c r="C267" s="4" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="D267" s="4" t="inlineStr"/>
+      <c r="E267" s="4" t="inlineStr"/>
+      <c r="F267" s="4" t="inlineStr"/>
+      <c r="G267" s="4" t="inlineStr"/>
+      <c r="H267" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I267" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J267" s="4" t="inlineStr"/>
+      <c r="K267" s="4" t="inlineStr"/>
+      <c r="L267" s="4" t="inlineStr"/>
+      <c r="M267" s="4" t="inlineStr"/>
+      <c r="N267" s="4" t="inlineStr"/>
+      <c r="O267" s="4" t="inlineStr"/>
+      <c r="P267" s="4" t="inlineStr">
+        <is>
+          <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="B268" s="4" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="C268" s="4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D268" s="4" t="inlineStr"/>
+      <c r="E268" s="4" t="inlineStr"/>
+      <c r="F268" s="4" t="inlineStr"/>
+      <c r="G268" s="4" t="inlineStr"/>
+      <c r="H268" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I268" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J268" s="4" t="inlineStr"/>
+      <c r="K268" s="4" t="inlineStr"/>
+      <c r="L268" s="4" t="inlineStr"/>
+      <c r="M268" s="4" t="inlineStr"/>
+      <c r="N268" s="4" t="inlineStr"/>
+      <c r="O268" s="4" t="inlineStr"/>
+      <c r="P268" s="4" t="inlineStr">
+        <is>
+          <t>Data fetch failed: Failed to fetch quote data after all retries</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="B269" s="4" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="C269" s="4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D269" s="4" t="inlineStr"/>
+      <c r="E269" s="4" t="inlineStr"/>
+      <c r="F269" s="4" t="inlineStr"/>
+      <c r="G269" s="4" t="inlineStr"/>
+      <c r="H269" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I269" s="4" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J269" s="4" t="inlineStr"/>
+      <c r="K269" s="4" t="inlineStr"/>
+      <c r="L269" s="4" t="inlineStr"/>
+      <c r="M269" s="4" t="inlineStr"/>
+      <c r="N269" s="4" t="inlineStr"/>
+      <c r="O269" s="4" t="inlineStr"/>
+      <c r="P269" s="4" t="inlineStr">
         <is>
           <t>Failed to fetch data: Failed to fetch quote data after all retries</t>
         </is>

</xml_diff>